<commit_message>
Align KD sam/visham with MVD generative/degenerative.
Replace leftover Chapter 1 *sam*/*visham* transliterations with generative/degenerative per MD-Mapping and MVD, and refresh the glossary note and PDFs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
+++ b/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
@@ -59827,7 +59827,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>KD 3.10: the three modes of गुण (property) — sam/visham matches the established sam-visham=generative-degenerative pairing (see सम विषम आवेश above); मध्यस्थ here is an adjective describing the property that maintains a composition once formed, distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
+          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
         </is>
       </c>
     </row>
@@ -62025,7 +62025,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KD 3.10: the three modes of गुण (property) — sam/visham matches the established sam-visham=generative-degenerative pairing (see सम विषम आवेश above); मध्यस्थ here is an adjective describing the property that maintains a composition once formed, distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
+          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
         </is>
       </c>
     </row>
@@ -62047,7 +62047,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KD 3.10: the three modes of गुण (property) — sam/visham matches the established sam-visham=generative-degenerative pairing (see सम विषम आवेश above); मध्यस्थ here is an adjective describing the property that maintains a composition once formed, distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
+          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise KD foreword and align progression/energised terms with MVD.
Rewrite the foreword opening sentence, replace leftover energy-endowed and awakening-sequence wording with MVD-aligned terms, and refresh the glossary and PDFs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
+++ b/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
@@ -58194,7 +58194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D148"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" style="114" min="1" max="1"/>
@@ -59196,1464 +59196,1464 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ग्राही</t>
+          <t>ऊर्जा सम्पन्न, पूर्णतया ऊर्जा सम्पन्न</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>grahi</t>
+          <t>urja sampanna</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>receptive</t>
+          <t>energised / fully energised</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>KD 3.13: all nature electricity-receptive</t>
+          <t>Aligned with MVD p.26 ("fully energised") and MD-Mapping ऊर्जित = Energised; supersedes earlier "energy-endowed". Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>विस्तार आयाम</t>
+          <t>ऊर्जा सम्पन्नता</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>vistār āyām</t>
+          <t>urja sampannata</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>energy-fullness</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>KD 3.14 chapter title; confirmed by Raghava (July 2026)</t>
+          <t>Per MD-Mapping; supersedes earlier "energy-endowment". Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>विस्तार</t>
+          <t>बल सम्पन्न, बल सम्पन्नता</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>vistār</t>
+          <t>bal sampanna / bal sampannata</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>extension (span)</t>
+          <t>forceful / forcefulness</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>KD 3.14: "whatever length, breadth, and height a composition is spread over"; distinct from the compound विस्तार आयाम \= area</t>
+          <t>Per MD-Mapping बल संपन्नता = Forcefulness; adjective parallel to energised. Supersedes earlier "force-endowed" / "force-endowment". Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>दृष्टि पाट</t>
+          <t>चुंबकीय बल सम्पन्न, चुंबकीय बल सम्पन्नता</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>drishti pat</t>
+          <t>chumbakiya bal sampanna / sampannata</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>span of vision</t>
+          <t>magnetic-force-full / magnetic force-fullness</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>KD 3.14: 90-degree binocular field</t>
+          <t>Per MD-Mapping चुंबकीय बल सम्पन्नता = magnetic force-fullness. Supersedes earlier "endowed with magnetic force" / "magnetic-force endowment". Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>दृग बिन्दु</t>
+          <t>ग्राही</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>drig bindu</t>
+          <t>grahi</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sight-point</t>
+          <t>receptive</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>KD 3.14</t>
+          <t>KD 3.13: all nature electricity-receptive</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>चक्षु तंत्र</t>
+          <t>विस्तार आयाम</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>chakshu tantra</t>
+          <t>vistār āyām</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>visual system</t>
+          <t>area</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>KD 3.14</t>
+          <t>KD 3.14 chapter title; confirmed by Raghava (July 2026)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>अंश (कोण में)</t>
+          <t>विस्तार</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ansh</t>
+          <t>vistār</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>degree (angle)</t>
+          <t>extension (span)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>KD 3.14 — same word as ansh=particle; sense depends on context</t>
+          <t>KD 3.14: "whatever length, breadth, and height a composition is spread over"; distinct from the compound विस्तार आयाम \= area</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>समकेन्द्रीय रेखा</t>
+          <t>दृष्टि पाट</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>samkendriya rekha</t>
+          <t>drishti pat</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>concentric line</t>
+          <t>span of vision</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>KD 3.14</t>
+          <t>KD 3.14: 90-degree binocular field</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>काल शून्य</t>
+          <t>दृग बिन्दु</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>kaal shoonya</t>
+          <t>drig bindu</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>time-zero</t>
+          <t>sight-point</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>KD 3.15</t>
+          <t>KD 3.14</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>घटी, पल</t>
+          <t>चक्षु तंत्र</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ghati, pal</t>
+          <t>chakshu tantra</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ghati, pal (time units)</t>
+          <t>visual system</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>KD 3.15, left transliterated</t>
+          <t>KD 3.14</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>फलन</t>
+          <t>अंश (कोण में)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>phalan</t>
+          <t>ansh</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>fruition</t>
+          <t>degree (angle)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>KD 3.15: evaluation on the basis of activity and fruition</t>
+          <t>KD 3.14 — same word as ansh=particle; sense depends on context</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>नित्य वर्तमान</t>
+          <t>समकेन्द्रीय रेखा</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>nitya vartman</t>
+          <t>samkendriya rekha</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ever-present</t>
+          <t>concentric line</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Settled per Raghava (July 2026); KD 3.15 predicate of kaal</t>
+          <t>KD 3.14</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>मेधस</t>
+          <t>काल शून्य</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>medhas</t>
+          <t>kaal shoonya</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>brain / medhas</t>
+          <t>time-zero</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>MD-Mapping: brain; KD 3.3 "medhas composition"</t>
+          <t>KD 3.15</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>शून्याकर्षण</t>
+          <t>घटी, पल</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>shunyakarshan</t>
+          <t>ghati, pal</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>zero-attraction</t>
+          <t>ghati, pal (time units)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>per MD-Mapping; KD 3.14</t>
+          <t>KD 3.15, left transliterated</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>परावर्तन</t>
+          <t>फलन</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>paravartan</t>
+          <t>phalan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>projection</t>
+          <t>fruition</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Re-settled per Raghava (2026-07-08), superseding the July 2026 KD-specific choice, to align with MD-Mapping's row, independently confirmed by MVD (MVD p.328). Ch. 3.12 retitled "Projection–Reflection"; all instances across KD-Karm-Darshan-English.md §3.11–3.12 and the confirmed paravartan instances in KD-Karm-Darshan-English.md §3.7–3.8 (heat-reflection passages, e.g. "the sun's heat is being projected equally in all directions") were swapped 2026-07-08</t>
+          <t>KD 3.15: evaluation on the basis of activity and fruition</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>प्रत्यावर्तन</t>
+          <t>नित्य वर्तमान</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>pratyavartan</t>
+          <t>nitya vartman</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>reflection</t>
+          <t>ever-present</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Re-settled per Raghava (2026-07-08), aligned with MD-Mapping/MVD (MVD p.286). See परावर्तन row above; swapped together as a pair 2026-07-08</t>
+          <t>Settled per Raghava (July 2026); KD 3.15 predicate of kaal</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>संसार (पशु/वनस्पति/खनिज-)</t>
+          <t>मेधस</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>sansar</t>
+          <t>medhas</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>order (animal order, plant order, mineral order, human order)</t>
+          <t>brain / medhas</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Per Raghava (July 2026): render -संसार compounds with "order," aligning with the four-orders vocabulary, not literal "world"</t>
+          <t>MD-Mapping: brain; KD 3.3 "medhas composition"</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>आत्मा, बुद्धि, चित्त, वृत्ति, मन</t>
+          <t>शून्याकर्षण</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>atma, buddhi, chitta, vritti, mun</t>
+          <t>shunyakarshan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>left transliterated (atma, buddhi, chitta, vritti, mun/"mind")</t>
+          <t>zero-attraction</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>KD 3.6: the five jeevan faculties (pūrvānukram), each carrying one of the five *sthiti* (state) activities — anubhav/atma (realisation), bodh/buddhi (enlightenment), chintan/chitta (contemplation), tulan/vritti (comparison), aswadan/mun (tasting) — and one of the five *gati* (motion) activities — praman/atma (evidence), ṛtambharā/buddhi (resoluteness), ichha/chitta (desire), vishleshan/vritti (analysis), chayan/mun (selection). MD-Mapping leaves all five untranslated; matches its own note under अंतर्नियामन ("पूर्वानुक्रम = वरीयता क्रम याने आत्मा, बुद्धि, चित्त, वृत्ति, मन")</t>
+          <t>per MD-Mapping; KD 3.14</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ऋतम्भरा, ऋतंभरा</t>
+          <t>परावर्तन</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ṛtambharā</t>
+          <t>paravartan</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>resoluteness</t>
+          <t>projection</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Per MD-Mapping; KD 3.4/3.6: buddhi's *gati* (motion) activity — putting justice, dharma, and truth to purpose and into practice</t>
+          <t>Re-settled per Raghava (2026-07-08), superseding the July 2026 KD-specific choice, to align with MD-Mapping's row, independently confirmed by MVD (MVD p.328). Ch. 3.12 retitled "Projection–Reflection"; all instances across KD-Karm-Darshan-English.md §3.11–3.12 and the confirmed paravartan instances in KD-Karm-Darshan-English.md §3.7–3.8 (heat-reflection passages, e.g. "the sun's heat is being projected equally in all directions") were swapped 2026-07-08</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>गठनपूर्णता, क्रियापूर्णता, आचरणपूर्णता</t>
+          <t>प्रत्यावर्तन</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>gathan-purnata, kriya-purnata, acharan-purnata</t>
+          <t>pratyavartan</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>constitutional completeness, activity-completeness, conduct-completeness</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>KD 3.3/3.4: the atom's three stages of development. गठनपूर्णता = "constitutional completeness" per MD-Mapping; क्रियापूर्णता and आचरणपूर्णता are parallel KD coinages (not in MD-Mapping), rendered analogously</t>
+          <t>Re-settled per Raghava (2026-07-08), aligned with MD-Mapping/MVD (MVD p.286). See परावर्तन row above; swapped together as a pair 2026-07-08</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>अखण्ड समाज</t>
+          <t>संसार (पशु/वनस्पति/खनिज-)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>akhand samaj</t>
+          <t>sansar</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>undivided society</t>
+          <t>order (animal order, plant order, mineral order, human order)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>KD 3.4: not in MD-Mapping; compositional rendering of अखण्ड (undivided) + समाज (society)</t>
+          <t>Per Raghava (July 2026): render -संसार compounds with "order," aligning with the four-orders vocabulary, not literal "world"</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>चिराकांक्षा, चिराकाँक्षा</t>
+          <t>आत्मा, बुद्धि, चित्त, वृत्ति, मन</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>chira-akanksha</t>
+          <t>atma, buddhi, chitta, vritti, mun</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>abiding aspiration</t>
+          <t>left transliterated (atma, buddhi, chitta, vritti, mun/"mind")</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>KD 3.6: not in MD-Mapping; judgment call — चिर (lasting/eternal) + आकांक्षा (aspiration/longing)</t>
+          <t>KD 3.6: the five jeevan faculties (pūrvānukram), each carrying one of the five *sthiti* (state) activities — anubhav/atma (realisation), bodh/buddhi (enlightenment), chintan/chitta (contemplation), tulan/vritti (comparison), aswadan/mun (tasting) — and one of the five *gati* (motion) activities — praman/atma (evidence), ṛtambharā/buddhi (resoluteness), ichha/chitta (desire), vishleshan/vritti (analysis), chayan/mun (selection). MD-Mapping leaves all five untranslated; matches its own note under अंतर्नियामन ("पूर्वानुक्रम = वरीयता क्रम याने आत्मा, बुद्धि, चित्त, वृत्ति, मन")</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>सचेष्ट</t>
+          <t>ऋतम्भरा, ऋतंभरा</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>sachesht</t>
+          <t>ṛtambharā</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>earnestly active</t>
+          <t>resoluteness</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>KD 3.6: not in MD-Mapping; judgment call for the state of alert, diligent striving toward the human goal</t>
+          <t>Per MD-Mapping; KD 3.4/3.6: buddhi's *gati* (motion) activity — putting justice, dharma, and truth to purpose and into practice</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>यथास्थिति</t>
+          <t>गठनपूर्णता, क्रियापूर्णता, आचरणपूर्णता</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>yatha-sthiti</t>
+          <t>gathan-purnata, kriya-purnata, acharan-purnata</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>actual condition</t>
+          <t>constitutional completeness, activity-completeness, conduct-completeness</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>KD 3.4/3.5: distinct from अस्तित्व (existence) — the concrete, as-is condition of a thing/person, not "status quo" in the political sense</t>
+          <t>KD 3.3/3.4: the atom's three stages of development. गठनपूर्णता = "constitutional completeness" per MD-Mapping; क्रियापूर्णता and आचरणपूर्णता are parallel KD coinages (not in MD-Mapping), rendered analogously</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>तृप्ति</t>
+          <t>अखण्ड समाज</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>tripti</t>
+          <t>akhand samaj</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>satiation</t>
+          <t>undivided society</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>KD 3.6: jeevan's fulfilment through realisation (*anubhav*), recognised in human tradition as happiness, peace, and contentment</t>
+          <t>KD 3.4: not in MD-Mapping; compositional rendering of अखण्ड (undivided) + समाज (society)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>परम</t>
+          <t>चिराकांक्षा, चिराकाँक्षा</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>param</t>
+          <t>chira-akanksha</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ultimate</t>
+          <t>abiding aspiration</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>KD 3.6: predicate of अनुभव (realisation) — "never more than realisation; jeevan remains incomplete in anything less"</t>
+          <t>KD 3.6: not in MD-Mapping; judgment call — चिर (lasting/eternal) + आकांक्षा (aspiration/longing)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ध्रुवीकरण</t>
+          <t>सचेष्ट</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>dhruvikaran</t>
+          <t>sachesht</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>anchoring</t>
+          <t>earnestly active</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("संतुलन स्वभाव गति"); KD 3.4: resolution becoming the fixed reference point of jeevan activity</t>
+          <t>KD 3.6: not in MD-Mapping; judgment call for the state of alert, diligent striving toward the human goal</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>गुण</t>
+          <t>यथास्थिति</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>guna</t>
+          <t>yatha-sthiti</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>actual condition</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08): "property," NOT "quality." MD-Mapping carries both readings (गुण = "properties" as a noun; गुण = "qualitative" as an adjective) — for KD's recurring रूप/गुण/स्वभाव/धर्म (form/property/essential nature/dharma) list of the four orders' predominant traits, and for chapter 3.10's title, गुण is a noun and takes "property." Retroactively corrected in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12, and KD-Karm-Darshan-English.md §3.13–3.15 (previously translated "quality") on 2026-07-08. Exception: the adjectival compound गुणात्मक परिवर्तन keeps MD-Mapping's own established "qualitative change/transformation" (KD 3.9) — "property-al" does not read in English, and MD-Mapping treats this compound as a separate row from bare गुण</t>
+          <t>KD 3.4/3.5: distinct from अस्तित्व (existence) — the concrete, as-is condition of a thing/person, not "status quo" in the political sense</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>सम, विषम, मध्यस्थ (गुण के रूप में)</t>
+          <t>तृप्ति</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>sam, visham, madhyastha</t>
+          <t>tripti</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>generative, degenerative, mediating</t>
+          <t>satiation</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
+          <t>KD 3.6: jeevan's fulfilment through realisation (*anubhav*), recognised in human tradition as happiness, peace, and contentment</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>सारक, मारक</t>
+          <t>परम</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>sarak(ta), marak(ta)</t>
+          <t>param</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>essential(ity), destructive(ness)</t>
+          <t>ultimate</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>KD 3.10: the two modes of स्वभाव (essential nature) in the prana state — sarakta = being abundant in itself and useful to the animal order; marakta = obstructing one's own seed-abundance and being disease/death-causing to the animal order</t>
+          <t>KD 3.6: predicate of अनुभव (realisation) — "never more than realisation; jeevan remains incomplete in anything less"</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>पात्रता</t>
+          <t>ध्रुवीकरण</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>patrata</t>
+          <t>dhruvikaran</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>worthiness</t>
+          <t>anchoring</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
+          <t>Per MD-Mapping ("संतुलन स्वभाव गति"); KD 3.4: resolution becoming the fixed reference point of jeevan activity</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>देव मानव, दिव्य मानव</t>
+          <t>गुण</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>dev manav, divya manav</t>
+          <t>guna</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>god-human, divine human</t>
+          <t>property</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>KD 3.10: literal rendering, judgment call; not in MD-Mapping</t>
+          <t>Settled per Raghava (2026-07-08): "property," NOT "quality." MD-Mapping carries both readings (गुण = "properties" as a noun; गुण = "qualitative" as an adjective) — for KD's recurring रूप/गुण/स्वभाव/धर्म (form/property/essential nature/dharma) list of the four orders' predominant traits, and for chapter 3.10's title, गुण is a noun and takes "property." Retroactively corrected in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12, and KD-Karm-Darshan-English.md §3.13–3.15 (previously translated "quality") on 2026-07-08. Exception: the adjectival compound गुणात्मक परिवर्तन keeps MD-Mapping's own established "qualitative change/transformation" (KD 3.9) — "property-al" does not read in English, and MD-Mapping treats this compound as a separate row from bare गुण</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>पशु मानव, राक्षस मानव</t>
+          <t>सम, विषम, मध्यस्थ (गुण के रूप में)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>pashu manav, rakshas manav</t>
+          <t>sam, visham, madhyastha</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>the animalistic human, the demonic human</t>
+          <t>generative, degenerative, mediating</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("animalistic human," "demonic human"). Retroactively corrected in KD-Karm-Darshan-English.md §3.9–3.10 on 2026-07-08 (previously "animal-human"/"demon-human") to match MD-Mapping exactly and align with KD 1's usage of the same pair</t>
+          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>राशि विधि</t>
+          <t>जागृति क्रम</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>rashi vidhi</t>
+          <t>jagriti kram</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>the arrangement of quantity</t>
+          <t>awakening progression</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>KD 3.9/3.10 closing line; not in MD-Mapping, compositional rendering (राशि = quantity/aggregate, विधि = method/arrangement)</t>
+          <t>Per MD-Mapping and MVD (not "awakening sequence"). Paired with विकास क्रम = development progression. Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>दृष्टा, ज्ञाता, ज्ञेय</t>
+          <t>विकास क्रम, विकासक्रम</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>drishta, gyata, gyeya</t>
+          <t>vikas kram</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>seer, knower, known</t>
+          <t>development progression</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Per MD-Mapping: दृष्टा=Seer, ज्ञाता=knower (not in PS), ज्ञेय=knowable (not in PS). KD 3.16-3.18 titles this triad "known" rather than MD-Mapping's literal "knowable" — reads more naturally as the object-pole of ज्ञान/ज्ञाता (knowledge/knower), a judgment call</t>
+          <t>Per MD-Mapping and MVD (not "developmental sequence"). Retroactively corrected remaining "developmental sequence" instances corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>कर्त्ता, भोक्ता</t>
+          <t>सारक, मारक</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>karta, bhokta</t>
+          <t>sarak(ta), marak(ta)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>doer, enjoyer</t>
+          <t>essential(ity), destructive(ness)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Compositional; कर्त्ता=doer (agent), भोक्ता=enjoyer (experiencer of result). KD 3.18 title</t>
+          <t>KD 3.10: the two modes of स्वभाव (essential nature) in the prana state — sarakta = being abundant in itself and useful to the animal order; marakta = obstructing one's own seed-abundance and being disease/death-causing to the animal order</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>दृश, दृश्य, दर्शन</t>
+          <t>पात्रता</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>drish, drishya, darshan</t>
+          <t>patrata</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>the seeing, the seen, seeing/philosophy</t>
+          <t>worthiness</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>KD 3.17: the seer-triad parallel to ज्ञान/ज्ञाता/ज्ञेय; left transliterated with bracketed gloss on first use, not in MD-Mapping under these exact senses</t>
+          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ध्यान, ध्याता, ध्येय</t>
+          <t>देव मानव, दिव्य मानव</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>dhyan, dhyata, dhyeya</t>
+          <t>dev manav, divya manav</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>attention, attender, object of attention</t>
+          <t>god-human, divine human</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>KD 3.17: not in MD-Mapping under this triad; compositional, parallel structure to ज्ञान/ज्ञाता/ज्ञेय</t>
+          <t>KD 3.10: literal rendering, judgment call; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>साध्य, साधक, साधन</t>
+          <t>पशु मानव, राक्षस मानव</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>sadhya, sadhak, sadhan</t>
+          <t>pashu manav, rakshas manav</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>aim, seeker, means</t>
+          <t>the animalistic human, the demonic human</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Per MD-Mapping: साध्य=aim, साधक=the seeker, साधन=the means. KD 3.17 triad</t>
+          <t>Per MD-Mapping ("animalistic human," "demonic human"). Retroactively corrected in KD-Karm-Darshan-English.md §3.9–3.10 on 2026-07-08 (previously "animal-human"/"demon-human") to match MD-Mapping exactly and align with KD 1's usage of the same pair</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>अध्यात्मवाद, अधिदैवीवाद, अधिभौतिकवाद</t>
+          <t>राशि विधि</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>adhyatmavad, adhidaivikvad, adhibhautikvad</t>
+          <t>rashi vidhi</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>spiritualism, god-centred-ism, materialism-of-the-beyond</t>
+          <t>the arrangement of quantity</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (kept close to transliteration: adhyatma-vada, Adhidaivika-vada, adhi-bhautikvad); KD 3.17 names the three classical schools collectively subsumed under आदर्शवाद (idealism)</t>
+          <t>KD 3.9/3.10 closing line; not in MD-Mapping, compositional rendering (राशि = quantity/aggregate, विधि = method/arrangement)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ब्रह्मवाद, आत्मवाद, जातिवाद, नस्लवाद, वंशवाद</t>
+          <t>दृष्टा, ज्ञाता, ज्ञेय</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>brahmavad, atmavad, jativad, naslvad, vanshvad</t>
+          <t>drishta, gyata, gyeya</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Brahma-doctrine, self-doctrine, casteism, racism, lineage-ism</t>
+          <t>seer, knower, known</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>KD 3.16: not in MD-Mapping, compositional renderings of the "-वाद" (doctrine/ism) compounds</t>
+          <t>Per MD-Mapping: दृष्टा=Seer, ज्ञाता=knower (not in PS), ज्ञेय=knowable (not in PS). KD 3.16-3.18 titles this triad "known" rather than MD-Mapping's literal "knowable" — reads more naturally as the object-pole of ज्ञान/ज्ञाता (knowledge/knower), a judgment call</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>उद्घाता</t>
+          <t>कर्त्ता, भोक्ता</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>udghata</t>
+          <t>karta, bhokta</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>herald</t>
+          <t>doer, enjoyer</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>KD 3.18: not in MD-Mapping, judgment call — the human being as the one who announces/evidences the awakened status</t>
+          <t>Compositional; कर्त्ता=doer (agent), भोक्ता=enjoyer (experiencer of result). KD 3.18 title</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>कर्म अभ्यास</t>
+          <t>दृश, दृश्य, दर्शन</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>karma abhyas</t>
+          <t>drish, drishya, darshan</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>practical-experiential method</t>
+          <t>the seeing, the seen, seeing/philosophy</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>KD 3.16: not in MD-Mapping under this compound; describes the Ayurveda/Unani diagnostic-treatment cycle (recognise disease → recognise medicine → treat, repeated until trust is earned)</t>
+          <t>KD 3.17: the seer-triad parallel to ज्ञान/ज्ञाता/ज्ञेय; left transliterated with bracketed gloss on first use, not in MD-Mapping under these exact senses</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>औकात</t>
+          <t>ध्यान, ध्याता, ध्येय</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>aukat</t>
+          <t>dhyan, dhyata, dhyeya</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>standing</t>
+          <t>attention, attender, object of attention</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>KD 3.16: colloquial Hindi/Urdu term for capacity/standing, not in MD-Mapping; KD uses it for the fixed capacity of human body-composition across generations</t>
+          <t>KD 3.17: not in MD-Mapping under this triad; compositional, parallel structure to ज्ञान/ज्ञाता/ज्ञेय</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>वेदना</t>
+          <t>साध्य, साधक, साधन</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>vedana</t>
+          <t>sadhya, sadhak, sadhan</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>pain</t>
+          <t>aim, seeker, means</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>KD 1: "the pressure of accepting the unacceptable — that itself is vedana." Not the same word as संवेदना (sensation/sensitivity, already established); matches MVD's own usage ("दूसरों के कष्ट, दुःख, वेदना... सुख" → "suffering, misery, pain... of others")</t>
+          <t>Per MD-Mapping: साध्य=aim, साधक=the seeker, साधन=the means. KD 3.17 triad</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>संचेतना</t>
+          <t>अध्यात्मवाद, अधिदैवीवाद, अधिभौतिकवाद</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>sanchetana</t>
+          <t>adhyatmavad, adhidaivikvad, adhibhautikvad</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>awareness</t>
+          <t>spiritualism, god-centred-ism, materialism-of-the-beyond</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), OVERRIDING MD-Mapping/SB's "Humane Consciousness" (SB Ch7 title) — "awareness" avoids collision with चेतना/जीव चेतना ("consciousness," e.g. "animal consciousness," KD 1) and चैतन्य ("conscious," e.g. "conscious activity," "material-conscious nature"), which stay untouched. Applies to संचेतनशील too ("awareness-endowed"). **Audit rule (2026-07-08 remediation):** grep for "human consciousness" / "higher-human consciousness" — replace with awareness / higher-awareness wherever the Hindi source is संचेतना; keep "consciousness" only for चेतना (e.g. "social consciousness" = सामाजिक चेतना, "consciousness-development" = चेतना विकास)</t>
+          <t>Per MD-Mapping (kept close to transliteration: adhyatma-vada, Adhidaivika-vada, adhi-bhautikvad); KD 3.17 names the three classical schools collectively subsumed under आदर्शवाद (idealism)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>अभीष्ट</t>
+          <t>ब्रह्मवाद, आत्मवाद, जातिवाद, नस्लवाद, वंशवाद</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>abhīṣṭa</t>
+          <t>brahmavad, atmavad, jativad, naslvad, vanshvad</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>desire</t>
+          <t>Brahma-doctrine, self-doctrine, casteism, racism, lineage-ism</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "desideratum" (itself an override of MD-Mapping's "Aim," chosen to avoid colliding with साध्य=aim). Note: this reintroduces a collision with इच्छा (the general term for desire throughout KD) — अभीष्ट and इच्छा are now both "desire" in English; distinguish by context if needed (अभीष्ट is the wished-for/happiness-directed sense, इच्छा the general faculty/act of desiring). साध्य keeps "aim." Where the source explicitly glosses one with the other ("साध्य (अभीष्ट)"), rendered as "the aim (the desire)"</t>
+          <t>KD 3.16: not in MD-Mapping, compositional renderings of the "-वाद" (doctrine/ism) compounds</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>कायिक</t>
+          <t>उद्घाता</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>kāyik</t>
+          <t>udghata</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>herald</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), aligning with MD-Mapping's own value ("physical," glossed "duty/responsibility carried out through the body together with mentality"), superseding this project's earlier "bodily" (chosen to avoid colliding with भौतिक=physical). Note: this reintroduces that collision — कायिक and भौतिक are now both "physical" in English; भौतिक is the material/physical-world sense (e.g. "physical substances," "physical science"), कायिक specifically the bodily-action sense in the कायिक/वाचिक/मानसिक (physical/vocal/mental) and "triad of behaviour" groupings — distinguish by context if needed</t>
+          <t>KD 3.18: not in MD-Mapping, judgment call — the human being as the one who announces/evidences the awakened status</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>कृत, कारित, अनुमोदित</t>
+          <t>कर्म अभ्यास</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>krit, karit, anumodit</t>
+          <t>karma abhyas</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>done, caused, intended</t>
+          <t>practical-experiential method</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "done, caused-to-be-done, and approved"/"consented-to." MD-Mapping's कृत="doing," कारित="getting done," अनुमोदित="consenting" — kept close but simplified; अनुमोदित specifically rendered "intended" rather than "approved"/"consenting" per this decision. Retrofitted in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances, including the related noun अनुमोदन→"intention") and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance) on 2026-07-08</t>
+          <t>KD 3.16: not in MD-Mapping under this compound; describes the Ayurveda/Unani diagnostic-treatment cycle (recognise disease → recognise medicine → treat, repeated until trust is earned)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>फल</t>
+          <t>औकात</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>phal</t>
+          <t>aukat</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>standing</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "fruit" — "phal means result of the action (karma)." Retrofitted in KD-Karm-Darshan-English.md on 2026-07-08 wherever फल stood alone (not फलन=fruition, not a फल-परिणाम compound, not literal fruit as food). See परिणाम for the resolved collision and the फल-परिणाम compound convention</t>
+          <t>KD 3.16: colloquial Hindi/Urdu term for capacity/standing, not in MD-Mapping; KD uses it for the fixed capacity of human body-composition across generations</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>परिणाम</t>
+          <t>वेदना</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>parinam</t>
+          <t>vedana</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>pain</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>REALIGNED 2026-07-08 with MVD/SB: श्रम-गति-परिणाम → "Effort – Motion – Result" (MVD/SB title-page Principle; MVD p.11). Both फल and bare परिणाम render as "result" in English — acceptable overlap where Hindi also overlaps (फल-परिणाम compounds collapse to "result" rather than "result-consequence"). Idiomatic connectors ("as a result of X") unchanged. Retrofitted corpus-wide across all 9 translation files on 2026-07-08 remediation pass</t>
+          <t>KD 1: "the pressure of accepting the unacceptable — that itself is vedana." Not the same word as संवेदना (sensation/sensitivity, already established); matches MVD's own usage ("दूसरों के कष्ट, दुःख, वेदना... सुख" → "suffering, misery, pain... of others")</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>अनुभूति</t>
+          <t>संचेतना</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>anubhūti</t>
+          <t>sanchetana</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>experiencing</t>
+          <t>awareness</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Judgment call, OVERRIDING MD-Mapping's "realisation" — MD-Mapping gives both अनुभूति and अनुभव as "realisation," but अनुभव is deeply entrenched across chapter 3 in KD-Karm-Darshan-English.md as "realisation" and the two words appear together/nearby throughout KD 1 (e.g. "सत्यानुभूति," "अनुभूति आनन्द"). अनुभव keeps "realisation"; अनुभूति becomes "experiencing" (the felt/sensed process) to keep them distinguishable</t>
+          <t>Settled per Raghava (2026-07-08), OVERRIDING MD-Mapping/SB's "Humane Consciousness" (SB Ch7 title) — "awareness" avoids collision with चेतना/जीव चेतना ("consciousness," e.g. "animal consciousness," KD 1) and चैतन्य ("conscious," e.g. "conscious activity," "material-conscious nature"), which stay untouched. Applies to संचेतनशील too ("awareness-endowed"). **Audit rule (2026-07-08 remediation):** grep for "human consciousness" / "higher-human consciousness" — replace with awareness / higher-awareness wherever the Hindi source is संचेतना; keep "consciousness" only for चेतना (e.g. "social consciousness" = सामाजिक चेतना, "consciousness-development" = चेतना विकास)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>सत्ता</t>
+          <t>अभीष्ट</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>sattā</t>
+          <t>abhīṣṭa</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Omnipotence</t>
+          <t>desire</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Per MD-Mapping. KD 1: the foundational basis of balance for all of nature ("अशेष प्रकृति का संतुलनाधार सत्ता ही है"); equated with अध्यात्म ("अध्यात्म (सत्ता) निरपेक्ष ज्ञान है")</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "desideratum" (itself an override of MD-Mapping's "Aim," chosen to avoid colliding with साध्य=aim). Note: this reintroduces a collision with इच्छा (the general term for desire throughout KD) — अभीष्ट and इच्छा are now both "desire" in English; distinguish by context if needed (अभीष्ट is the wished-for/happiness-directed sense, इच्छा the general faculty/act of desiring). साध्य keeps "aim." Where the source explicitly glosses one with the other ("साध्य (अभीष्ट)"), rendered as "the aim (the desire)"</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>अध्यात्म</t>
+          <t>कायिक</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>adhyātma</t>
+          <t>kāyik</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>the Spirit</t>
+          <t>physical</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("The Spirit"). KD 1: "जड़-चैतन्यात्मक प्रकृति की आधारपूर्ण सत्ता ही अध्यात्म है" — glossed in-text as equivalent to सत्ता (Omnipotence), rendered "the Spirit (Omnipotence)" on first use</t>
+          <t>Settled per Raghava (2026-07-08), aligning with MD-Mapping's own value ("physical," glossed "duty/responsibility carried out through the body together with mentality"), superseding this project's earlier "bodily" (chosen to avoid colliding with भौतिक=physical). Note: this reintroduces that collision — कायिक and भौतिक are now both "physical" in English; भौतिक is the material/physical-world sense (e.g. "physical substances," "physical science"), कायिक specifically the bodily-action sense in the कायिक/वाचिक/मानसिक (physical/vocal/mental) and "triad of behaviour" groupings — distinguish by context if needed</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>संस्कार</t>
+          <t>कृत, कारित, अनुमोदित</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>sanskar</t>
+          <t>krit, karit, anumodit</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>*sanskar* (left transliterated)</t>
+          <t>done, caused, intended</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (kept as "Sanskar," not translated). Settled per this project (2026-07-08): KD 1 uses संस्कार and संस्कृति together constantly (e.g. "संस्कार, संस्कृति व सभ्यता") — collapsing both to "culture" erases the distinction. संस्कार = the individual's cultural conditioning/refinement (kept as *sanskar*); संस्कृति = the collective/civilizational achievement (kept as "culture"); सभ्यता = "civilisation"</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "done, caused-to-be-done, and approved"/"consented-to." MD-Mapping's कृत="doing," कारित="getting done," अनुमोदित="consenting" — kept close but simplified; अनुमोदित specifically rendered "intended" rather than "approved"/"consenting" per this decision. Retrofitted in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances, including the related noun अनुमोदन→"intention") and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance) on 2026-07-08</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>संस्कृति</t>
+          <t>फल</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>sanskriti</t>
+          <t>phal</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>culture</t>
+          <t>result</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>See संस्कार above — kept distinct from it. सुसंस्कृति = "wholesome culture," विकृत संस्कृति = "corrupted culture"</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "fruit" — "phal means result of the action (karma)." Retrofitted in KD-Karm-Darshan-English.md on 2026-07-08 wherever फल stood alone (not फलन=fruition, not a फल-परिणाम compound, not literal fruit as food). See परिणाम for the resolved collision and the फल-परिणाम compound convention</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>सभ्यता</t>
+          <t>परिणाम</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>sabhyata</t>
+          <t>parinam</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>civilisation</t>
+          <t>result</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("civilization, civility")</t>
+          <t>REALIGNED 2026-07-08 with MVD/SB: श्रम-गति-परिणाम → "Effort – Motion – Result" (MVD/SB title-page Principle; MVD p.11). Both फल and bare परिणाम render as "result" in English — acceptable overlap where Hindi also overlaps (फल-परिणाम compounds collapse to "result" rather than "result-consequence"). Idiomatic connectors ("as a result of X") unchanged. Retrofitted corpus-wide across all 9 translation files on 2026-07-08 remediation pass</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>काम</t>
+          <t>अनुभूति</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>kama</t>
+          <t>anubhūti</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>*kama* (desire)</t>
+          <t>experiencing</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>KD 1: contextual exception — MD-Mapping's "lust" is too narrow for the classical चतुर्वर्ग (मोक्ष/धर्म/काम/अर्थ) listing, where काम denotes desire/pleasure as a life-aim, not specifically sexual desire. Left transliterated with gloss "(desire)" on first use, distinct from इच्छा (the general term for desire throughout KD)</t>
+          <t>Judgment call, OVERRIDING MD-Mapping's "realisation" — MD-Mapping gives both अनुभूति and अनुभव as "realisation," but अनुभव is deeply entrenched across chapter 3 in KD-Karm-Darshan-English.md as "realisation" and the two words appear together/nearby throughout KD 1 (e.g. "सत्यानुभूति," "अनुभूति आनन्द"). अनुभव keeps "realisation"; अनुभूति becomes "experiencing" (the felt/sensed process) to keep them distinguishable</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>अर्थ</t>
+          <t>सत्ता</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>artha</t>
+          <t>sattā</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>wealth (contextual)</t>
+          <t>Omnipotence</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("resources"), rendered "wealth" for readability in the चतुर्वर्ग list and wealth/resource contexts ("अर्थ तन, मन, धन है"). CONTEXTUAL EXCEPTION: where अर्थ is used epistemically (e.g. "सम्पूर्ण अर्थ का पूर्ण अर्थ अनुभव ही है"), it means "meaning," not "wealth" — judge from context</t>
+          <t>Per MD-Mapping. KD 1: the foundational basis of balance for all of nature ("अशेष प्रकृति का संतुलनाधार सत्ता ही है"); equated with अध्यात्म ("अध्यात्म (सत्ता) निरपेक्ष ज्ञान है")</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>कासा, आकूति, मेधा</t>
+          <t>अध्यात्म</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>kāsā, ākūti, medhā</t>
+          <t>adhyātma</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>left transliterated</t>
+          <t>the Spirit</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>KD 1: an obscure classical triad of "union-born intellect" (योग-जन्य-बुद्धि), not in MD-Mapping. Glossed in-text on first occurrence (poet/sage-artist; divine worker; divine knower with complete knowledge) — judgment call, flag for review against a Sanskrit dictionary if precision matters</t>
+          <t>Per MD-Mapping ("The Spirit"). KD 1: "जड़-चैतन्यात्मक प्रकृति की आधारपूर्ण सत्ता ही अध्यात्म है" — glossed in-text as equivalent to सत्ता (Omnipotence), rendered "the Spirit (Omnipotence)" on first use</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>मति, सुमति, अनुमति</t>
+          <t>संस्कार</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>mati, sumati, anumati</t>
+          <t>sanskar</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>left transliterated</t>
+          <t>*sanskar* (left transliterated)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>KD 1: triad of "righteous-action-born intellect" (सुकर्म-जन्य-बुद्धि), not in MD-Mapping; left transliterated, glossed in-text</t>
+          <t>Per MD-Mapping (kept as "Sanskar," not translated). Settled per this project (2026-07-08): KD 1 uses संस्कार and संस्कृति together constantly (e.g. "संस्कार, संस्कृति व सभ्यता") — collapsing both to "culture" erases the distinction. संस्कार = the individual's cultural conditioning/refinement (kept as *sanskar*); संस्कृति = the collective/civilizational achievement (kept as "culture"); सभ्यता = "civilisation"</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>अमति, कुमति, दुर्मति</t>
+          <t>संस्कृति</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>amati, kumati, durmati</t>
+          <t>sanskriti</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>left transliterated</t>
+          <t>culture</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>KD 1: triad of "unrighteous-action-born tendency" (दुष्कर्म-जन्य-प्रवृत्ति), parallel to मति/सुमति/अनुमति; not in MD-Mapping</t>
+          <t>See संस्कार above — kept distinct from it. सुसंस्कृति = "wholesome culture," विकृत संस्कृति = "corrupted culture"</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>निवृत्ति</t>
+          <t>सभ्यता</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>nivṛtti</t>
+          <t>sabhyata</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>disencumberance</t>
+          <t>civilisation</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
+          <t>Per MD-Mapping ("civilization, civility")</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>संवेग</t>
+          <t>काम</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>samveg</t>
+          <t>kama</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>impetus</t>
+          <t>*kama* (desire)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Per MD-Mapping</t>
+          <t>KD 1: contextual exception — MD-Mapping's "lust" is too narrow for the classical चतुर्वर्ग (मोक्ष/धर्म/काम/अर्थ) listing, where काम denotes desire/pleasure as a life-aim, not specifically sexual desire. Left transliterated with gloss "(desire)" on first use, distinct from इच्छा (the general term for desire throughout KD)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>पुण्यात्मा, पापात्मा</t>
+          <t>अर्थ</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>punyatma, papatma</t>
+          <t>artha</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>the meritorious soul, the sinful soul</t>
+          <t>wealth (contextual)</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>KD 1: not in MD-Mapping as a pair; compositional (पुण्य=merit, पाप=sin, आत्मा=soul), paired with सुखी/दुखी (happy/unhappy) across the five states (individual/family/society/nation/international)</t>
+          <t>Per MD-Mapping ("resources"), rendered "wealth" for readability in the चतुर्वर्ग list and wealth/resource contexts ("अर्थ तन, मन, धन है"). CONTEXTUAL EXCEPTION: where अर्थ is used epistemically (e.g. "सम्पूर्ण अर्थ का पूर्ण अर्थ अनुभव ही है"), it means "meaning," not "wealth" — judge from context</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>स्थूल, सूक्ष्म, कारण</t>
+          <t>कासा, आकूति, मेधा</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>sthula, sukshma, karana</t>
+          <t>kāsā, ākūti, medhā</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>gross, subtle, causal</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
+          <t>KD 1: an obscure classical triad of "union-born intellect" (योग-जन्य-बुद्धि), not in MD-Mapping. Glossed in-text on first occurrence (poet/sage-artist; divine worker; divine knower with complete knowledge) — judgment call, flag for review against a Sanskrit dictionary if precision matters</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>रजोगुण, तमोगुण, सत्वगुण</t>
+          <t>मति, सुमति, अनुमति</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>rajoguna, tamoguna, sattvaguna</t>
+          <t>mati, sumati, anumati</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -60663,797 +60663,929 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>KD 1: the classical three गुण (property-modes), mapped onto sam/visham/mediating (see सम-विषम-मध्यस्थ row above: sam=rajoguna, visham=tamoguna, mediating=sattvaguna); not in MD-Mapping, kept transliterated per standard practice for this well-known Sanskrit triad</t>
+          <t>KD 1: triad of "righteous-action-born intellect" (सुकर्म-जन्य-बुद्धि), not in MD-Mapping; left transliterated, glossed in-text</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>नियम-त्रय, व्यवहार-त्रय, अन्वेषण-त्रय</t>
+          <t>अमति, कुमति, दुर्मति</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>niyam-tray, vyavahar-tray, anveshan-tray</t>
+          <t>amati, kumati, durmati</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>triad of rule, triad of behaviour, triad of investigation</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>KD 1: compositional (X-त्रय = "triad of X"); niyam-tray = intellectual/social/natural rule, vyavahar-tray = physical/vocal/mental behaviour, anveshan-tray = object-/desire-/truth-investigation</t>
+          <t>KD 1: triad of "unrighteous-action-born tendency" (दुष्कर्म-जन्य-प्रवृत्ति), parallel to मति/सुमति/अनुमति; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>मानवीयतापूर्ण (X) / अतिमानवीयतापूर्ण (X)</t>
+          <t>निवृत्ति</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>manviyatapurna, atimanviyatapurna</t>
+          <t>nivṛtti</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>humane (X) / higher-humane (X)</t>
+          <t>disencumberance</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>CORRECTION, 2026-07-08: MD-Mapping has direct rows मानवीयता पूर्ण आचरण = "Humane Conduct" and मानवीयता पूर्ण आचरण ज्ञान = "knowledge of humane conduct." MVD independently confirms in running prose: "...जीवन ज्ञान व मानवीयतापूर्ण आचरण ज्ञान..." → "...knowledge of jeevan and humane conduct" (MVD p.3); MVD also has a dedicated glossary entry "मानवीयतापूर्ण व्यवहार" → "Humane Behaviour" (MVD p.34). The "X-पूर्ण" suffix (X-filled/X-replete) is therefore a plain adjective in English ("humane"), not "conduct filled with humaneness" or "humaneness-replete conduct." Retrofitted in KD-Karm-Darshan-English.md (ch. 2) (7 instances) and KD-Karm-Darshan-English.md (ch. 1) (~15 instances, verified against source images pp.8, 9, 10, 11, 16, 18, 24, 28) on 2026-07-08, wherever मानवीयतापूर्ण/अतिमानवीयतापूर्ण directly modified a noun (आचरण, व्यवहार, स्वभाव, मानव, कार्यक्रम, पद्धति, etc.). Not touched: bare मानवीयता/अतिमानवीयता used as nouns ("in humaneness and higher-humaneness"), and unrelated "-पूर्ण" compounds on other roots (e.g. सत्यतापूर्ण = "truthfulness-replete," सहअस्तित्व-replete, ज्ञान-/विवेक-/विज्ञान-पूर्ण = "knowledge-/wisdom-/science-filled" — different words, out of scope for this correction). **CHAPTER 3 SWEEP, 2026-07-08:** the same "X-replete-with-humaneness"/"humanity-replete X" error (variant wordings of the same underlying मानवीयतापूर्ण mistranslation) was also found and fixed across chapter 3: KD-Karm-Darshan-English.md §3.4–3.6 (2 instances, including one inside the recurring three-part knowledge formula — see जीवन ज्ञान row), KD-Karm-Darshan-English.md §3.9–3.10 (4 instances, using "humanity-replete" rather than "humaneness-replete"), and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance, inside the same three-part formula). KD-Karm-Darshan-English.md §3.1–3.3, KD-Karm-Darshan-English.md §3.7–3.8, and KD-Karm-Darshan-English.md §3.13–3.15 had no instances of this error</t>
+          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>जीवन ज्ञान</t>
+          <t>संवेग</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>jeevan gyan</t>
+          <t>samveg</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>knowledge of jeevan</t>
+          <t>impetus</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>CORRECTION, 2026-07-08: MVD confirms "जीवन ज्ञान" → "knowledge of jeevan" in both instances of the recurring three-part formula (अस्तित्व दर्शन ज्ञान / जीवन ज्ञान / मानवीयतापूर्ण आचरण ज्ञान): "...जीवन ज्ञान व मानवीयतापूर्ण आचरण ज्ञान..." → "...knowledge of jeevan and humane conduct" (MVD p.3), and "...चैतन्य प्रकृति रूपी जीवन ज्ञान..." → "...knowledge of jeevan in the form of sentient nature..." (MVD p.259). Keeps the "knowledge of X" pattern parallel across all three terms, matching the established renderings of the other two (see दर्शन and मानवीयतापूर्ण rows above/below). Retrofitted in KD-Karm-Darshan-English.md (ch. 2)'s opening line (had "jeevan knowledge") on 2026-07-08. Also retrofitted across all of chapter 3 on 2026-07-08 (see चैप्टर 3 sweep note under the मानवीयतापूर्ण row): "jeevan-knowledge"/"jeevan knowledge" → "the knowledge of jeevan" in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12 (×2), and KD-Karm-Darshan-English.md §3.16–3.18 (×2); "darshan-knowledge" and bare "darshan" (in the same non-triad, non-proper-noun sense) → "the knowledge of the holistic view"/"the holistic view" in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances)</t>
+          <t>Per MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>गम्यता</t>
+          <t>पुण्यात्मा, पापात्मा</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>gamyata</t>
+          <t>punyatma, papatma</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>the destination</t>
+          <t>the meritorious soul, the sinful soul</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>KD 1: abstract-noun form of गम्य/गन्तव्य (already "destination" per KD 3.12/3.14 glossary row); not in MD-Mapping, treated as the same concept</t>
+          <t>KD 1: not in MD-Mapping as a pair; compositional (पुण्य=merit, पाप=sin, आत्मा=soul), paired with सुखी/दुखी (happy/unhappy) across the five states (individual/family/society/nation/international)</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>दर्शन (bare, or in "X दर्शन ज्ञान" / "X दर्शन" / "दर्शन-क्षमता" compounds)</t>
+          <t>स्थूल, सूक्ष्म, कारण</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>darshan</t>
+          <t>sthula, sukshma, karana</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>the holistic view (of X)</t>
+          <t>gross, subtle, causal</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>CORRECTION, 2026-07-08: MD-Mapping has a direct row for bare दर्शन = "Holistic view, Worldview, Philosophy," plus confirmed compound rows सह-अस्तित्व दर्शन ज्ञान = "knowledge of holistic view of coexistence" and मानव कर्म दर्शन (this book's own title) = "Holistic view of Human Action." MVD independently confirms the exact KD 2 phrase: "अस्तित्व दर्शन ज्ञान" → "knowledge of the holistic view of existence" (MVD p.259, near-verbatim to KD 2's opening line). Retrofitted in KD-Karm-Darshan-English.md (ch. 2) (4 instances: the opening "अस्तित्व दर्शन ज्ञान," "(पूर्ण-दर्शन)," and two "दर्शन-क्षमता" instances) and in KD-Karm-Darshan-English.md (ch. 1) (10 instances, verified page-by-page against the source images: pp.1, 3, 13, 14, 15 (×2), 16 (×2 continuing to 17), 17 (×2)) on 2026-07-08. Excluded from this correction (kept as-is): the proper noun "Madhyasth Darshan" (book/philosophy name, p.19, always transliterated); the दृश/दृश्य/दर्शन seer-triad sense (KD 3.17, see separate row below, a distinct established convention); and the verbal usage "X का दर्शन करना" = "to behold X" (KD 1 p.24, four instances, e.g. "vritti... beholds the mind" — this is the common devotional-register verb "to behold/have sight of," not the noun "holistic view," and one redundant instance ("beholds the darshan of the less-awakened") was simplified to "beholds the less-awakened" accordingly</t>
+          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>उपासना</t>
+          <t>रजोगुण, तमोगुण, सत्वगुण</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>upāsanā</t>
+          <t>rajoguna, tamoguna, sattvaguna</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Upasana (worship)</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
+          <t>KD 1: the classical three गुण (property-modes), mapped onto sam/visham/mediating (see सम-विषम-मध्यस्थ row above: sam=rajoguna, visham=tamoguna, mediating=sattvaguna); not in MD-Mapping, kept transliterated per standard practice for this well-known Sanskrit triad</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>विवेक</t>
+          <t>नियम-त्रय, व्यवहार-त्रय, अन्वेषण-त्रय</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>vivek</t>
+          <t>niyam-tray, vyavahar-tray, anveshan-tray</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>wisdom</t>
+          <t>triad of rule, triad of behaviour, triad of investigation</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("wisdom"); KD 2 chapter subtitle ("उपासना – विवेक" → "Upasana – Wisdom")</t>
+          <t>KD 1: compositional (X-त्रय = "triad of X"); niyam-tray = intellectual/social/natural rule, vyavahar-tray = physical/vocal/mental behaviour, anveshan-tray = object-/desire-/truth-investigation</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>नश्वरत्व</t>
+          <t>मानवीयतापूर्ण (X) / अतिमानवीयतापूर्ण (X)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>nashwaratva</t>
+          <t>manviyatapurna, atimanviyatapurna</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>perishability</t>
+          <t>humane (X) / higher-humane (X)</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
+          <t>CORRECTION, 2026-07-08: MD-Mapping has direct rows मानवीयता पूर्ण आचरण = "Humane Conduct" and मानवीयता पूर्ण आचरण ज्ञान = "knowledge of humane conduct." MVD independently confirms in running prose: "...जीवन ज्ञान व मानवीयतापूर्ण आचरण ज्ञान..." → "...knowledge of jeevan and humane conduct" (MVD p.3); MVD also has a dedicated glossary entry "मानवीयतापूर्ण व्यवहार" → "Humane Behaviour" (MVD p.34). The "X-पूर्ण" suffix (X-filled/X-replete) is therefore a plain adjective in English ("humane"), not "conduct filled with humaneness" or "humaneness-replete conduct." Retrofitted in KD-Karm-Darshan-English.md (ch. 2) (7 instances) and KD-Karm-Darshan-English.md (ch. 1) (~15 instances, verified against source images pp.8, 9, 10, 11, 16, 18, 24, 28) on 2026-07-08, wherever मानवीयतापूर्ण/अतिमानवीयतापूर्ण directly modified a noun (आचरण, व्यवहार, स्वभाव, मानव, कार्यक्रम, पद्धति, etc.). Not touched: bare मानवीयता/अतिमानवीयता used as nouns ("in humaneness and higher-humaneness"), and unrelated "-पूर्ण" compounds on other roots (e.g. सत्यतापूर्ण = "truthfulness-replete," सहअस्तित्व-replete, ज्ञान-/विवेक-/विज्ञान-पूर्ण = "knowledge-/wisdom-/science-filled" — different words, out of scope for this correction). **CHAPTER 3 SWEEP, 2026-07-08:** the same "X-replete-with-humaneness"/"humanity-replete X" error (variant wordings of the same underlying मानवीयतापूर्ण mistranslation) was also found and fixed across chapter 3: KD-Karm-Darshan-English.md §3.4–3.6 (2 instances, including one inside the recurring three-part knowledge formula — see जीवन ज्ञान row), KD-Karm-Darshan-English.md §3.9–3.10 (4 instances, using "humanity-replete" rather than "humaneness-replete"), and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance, inside the same three-part formula). KD-Karm-Darshan-English.md §3.1–3.3, KD-Karm-Darshan-English.md §3.7–3.8, and KD-Karm-Darshan-English.md §3.13–3.15 had no instances of this error</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>कूटस्थ, रूपस्थ, आत्मस्थ (उपासना के रूप में)</t>
+          <t>जीवन ज्ञान</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>kutastha, rupastha, atmastha</t>
+          <t>jeevan gyan</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>kutastha upasana (abiding in the immutable), rupastha upasana (abiding in form), atmastha upasana (abiding in the self)</t>
+          <t>knowledge of jeevan</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>KD 2: the three loci/modes of upasana (undertaken respectively for complete realisation; for proximity to a form together with magnificence; and as the process of reflection/*pratyavartan*). Not in MD-Mapping; left transliterated with compositional glosses, judgment call</t>
+          <t>CORRECTION, 2026-07-08: MVD confirms "जीवन ज्ञान" → "knowledge of jeevan" in both instances of the recurring three-part formula (अस्तित्व दर्शन ज्ञान / जीवन ज्ञान / मानवीयतापूर्ण आचरण ज्ञान): "...जीवन ज्ञान व मानवीयतापूर्ण आचरण ज्ञान..." → "...knowledge of jeevan and humane conduct" (MVD p.3), and "...चैतन्य प्रकृति रूपी जीवन ज्ञान..." → "...knowledge of jeevan in the form of sentient nature..." (MVD p.259). Keeps the "knowledge of X" pattern parallel across all three terms, matching the established renderings of the other two (see दर्शन and मानवीयतापूर्ण rows above/below). Retrofitted in KD-Karm-Darshan-English.md (ch. 2)'s opening line (had "jeevan knowledge") on 2026-07-08. Also retrofitted across all of chapter 3 on 2026-07-08 (see चैप्टर 3 sweep note under the मानवीयतापूर्ण row): "jeevan-knowledge"/"jeevan knowledge" → "the knowledge of jeevan" in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12 (×2), and KD-Karm-Darshan-English.md §3.16–3.18 (×2); "darshan-knowledge" and bare "darshan" (in the same non-triad, non-proper-noun sense) → "the knowledge of the holistic view"/"the holistic view" in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances)</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>देवात्मा, भूतात्मा, दिव्यात्मा</t>
+          <t>गम्यता</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>devatma, bhootatma, divyatma</t>
+          <t>gamyata</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>the deific soul, the elemental soul, the divine soul</t>
+          <t>the destination</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+          <t>KD 1: abstract-noun form of गम्य/गन्तव्य (already "destination" per KD 3.12/3.14 glossary row); not in MD-Mapping, treated as the same concept</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>जीवन-पुंज</t>
+          <t>दर्शन (bare, or in "X दर्शन ज्ञान" / "X दर्शन" / "दर्शन-क्षमता" compounds)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>jeevan-punj</t>
+          <t>darshan</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>jeevan-cluster</t>
+          <t>the holistic view (of X)</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>KD 2: "the conscious unit is the combined form of subtle and causal activity; this itself is the jeevan-punj" — not in MD-Mapping, compositional (पुंज = cluster/mass)</t>
+          <t>CORRECTION, 2026-07-08: MD-Mapping has a direct row for bare दर्शन = "Holistic view, Worldview, Philosophy," plus confirmed compound rows सह-अस्तित्व दर्शन ज्ञान = "knowledge of holistic view of coexistence" and मानव कर्म दर्शन (this book's own title) = "Holistic view of Human Action." MVD independently confirms the exact KD 2 phrase: "अस्तित्व दर्शन ज्ञान" → "knowledge of the holistic view of existence" (MVD p.259, near-verbatim to KD 2's opening line). Retrofitted in KD-Karm-Darshan-English.md (ch. 2) (4 instances: the opening "अस्तित्व दर्शन ज्ञान," "(पूर्ण-दर्शन)," and two "दर्शन-क्षमता" instances) and in KD-Karm-Darshan-English.md (ch. 1) (10 instances, verified page-by-page against the source images: pp.1, 3, 13, 14, 15 (×2), 16 (×2 continuing to 17), 17 (×2)) on 2026-07-08. Excluded from this correction (kept as-is): the proper noun "Madhyasth Darshan" (book/philosophy name, p.19, always transliterated); the दृश/दृश्य/दर्शन seer-triad sense (KD 3.17, see separate row below, a distinct established convention); and the verbal usage "X का दर्शन करना" = "to behold X" (KD 1 p.24, four instances, e.g. "vritti... beholds the mind" — this is the common devotional-register verb "to behold/have sight of," not the noun "holistic view," and one redundant instance ("beholds the darshan of the less-awakened") was simplified to "beholds the less-awakened" accordingly</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>विषय-चतुष्टय, चतुर्विषय</t>
+          <t>उपासना</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>vishaya-chatushtaya</t>
+          <t>upāsanā</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>instincts-quad / the four-object domain</t>
+          <t>Upasana (worship)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("विषय चतुष्टय = instincts-quad"). KD 2 uses both विषय-चतुष्टय and the equivalent चतुर्विषय; both rendered with the same established English</t>
+          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ऐषणा-त्रय</t>
+          <t>विवेक</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>eshana-traya</t>
+          <t>vivek</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>the triad of desires</t>
+          <t>wisdom</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>KD 2: paired with विषय-चतुष्टय, tied to adhidaivik (social/behavioural) values. Not in MD-Mapping; left transliterated per the classical Sanskrit ऐषणा-त्रय (putra/vitta/loka-eshana), judgment call</t>
+          <t>Per MD-Mapping ("wisdom"); KD 2 chapter subtitle ("उपासना – विवेक" → "Upasana – Wisdom")</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>विद्या, उपविद्या, क्षुद्र विद्या</t>
+          <t>नश्वरत्व</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>vidya, upavidya, kshudra vidya</t>
+          <t>nashwaratva</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>learning, sub-learning, base learning</t>
+          <t>perishability</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
+          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>नियम-त्रय</t>
+          <t>कूटस्थ, रूपस्थ, आत्मस्थ (उपासना के रूप में)</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>niyam-tray</t>
+          <t>kutastha, rupastha, atmastha</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>the "triad of rule"</t>
+          <t>kutastha upasana (abiding in the immutable), rupastha upasana (abiding in form), atmastha upasana (abiding in the self)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Reused from KD 1 (see निवृत्ति-area rows below and KD-3 glossary); KD 2 explicitly glosses it as "बौद्धिक, सामाजिक एवं प्राकृतिक" (intellectual, social, and natural), confirming the KD 1 gloss</t>
+          <t>KD 2: the three loci/modes of upasana (undertaken respectively for complete realisation; for proximity to a form together with magnificence; and as the process of reflection/*pratyavartan*). Not in MD-Mapping; left transliterated with compositional glosses, judgment call</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>जागृति-त्रय, शक्ति-त्रय</t>
+          <t>देवात्मा, भूतात्मा, दिव्यात्मा</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>jagriti-traya, shakti-traya</t>
+          <t>devatma, bhootatma, divyatma</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>the "triad of awakening", the "triad of powers"</t>
+          <t>the deific soul, the elemental soul, the divine soul</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>KD 2: new parallel formations on the established "-त्रय = triad of X" pattern (see नियम-त्रय, व्यवहार-त्रय, अन्वेषण-त्रय, KD 1 glossary row). जागृति-त्रय = awakening of इच्छा/क्रिया/ज्ञान शक्ति (desire-, activity-, and knowledge-power); शक्ति-त्रय = the same three powers named directly</t>
+          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>इच्छा शक्ति, क्रिया शक्ति, ज्ञान शक्ति</t>
+          <t>जीवन-पुंज</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ichha shakti, kriya shakti, gyan shakti</t>
+          <t>jeevan-punj</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>desire-power, activity-power, knowledge-power</t>
+          <t>jeevan-cluster</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>KD 2: classical triad (kriya-shakti/iccha-shakti/jnana-shakti); not in MD-Mapping under this grouping, compositional</t>
+          <t>KD 2: "the conscious unit is the combined form of subtle and causal activity; this itself is the jeevan-punj" — not in MD-Mapping, compositional (पुंज = cluster/mass)</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ता-त्रय</t>
+          <t>विषय-चतुष्टय, चतुर्विषय</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>tā-traya</t>
+          <t>vishaya-chatushtaya</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>the "triad of *-tā*"</t>
+          <t>instincts-quad / the four-object domain</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>KD 2 p.44: "स्वयं का मूल्यांकन 'ता-त्रय' की सीमा में होता है" (self-evaluation occurs within the domain of the tā-traya). UNCERTAIN — not in MD-Mapping; the surrounding text repeatedly pairs क्षमता/योग्यता/पात्रता (capacity/competence/worthiness), which is the likeliest referent, but the source does not gloss the compound explicitly here. Left transliterated and flagged for human review rather than asserted</t>
+          <t>Per MD-Mapping ("विषय चतुष्टय = instincts-quad"). KD 2 uses both विषय-चतुष्टय and the equivalent चतुर्विषय; both rendered with the same established English</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>अनुक्षण-विक्षण-वृत्ति, सहजावृत्ति</t>
+          <t>ऐषणा-त्रय</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>anukshan-vikshan-vritti, sahajavritti</t>
+          <t>eshana-traya</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>the moment-to-moment unbroken tendency; natural-recurrence</t>
+          <t>the triad of desires</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>KD 2 p.43/45: defined in-text as "the disappearance of moment-to-moment mediating obstruction." Not in MD-Mapping; compositional, glossed in-text on first use</t>
+          <t>KD 2: paired with विषय-चतुष्टय, tied to adhidaivik (social/behavioural) values. Not in MD-Mapping; left transliterated per the classical Sanskrit ऐषणा-त्रय (putra/vitta/loka-eshana), judgment call</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>तदाकार</t>
+          <t>विद्या, उपविद्या, क्षुद्र विद्या</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>tadakar</t>
+          <t>vidya, upavidya, kshudra vidya</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>taking-the-form-of</t>
+          <t>learning, sub-learning, base learning</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
+          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>सम्यक्-बोध, सम्यक् संकल्प</t>
+          <t>नियम-त्रय</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>samyak-bodh, samyak sankalp</t>
+          <t>niyam-tray</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>right-enlightenment, right resolve</t>
+          <t>the "triad of rule"</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>KD 2: सम्यक् = classical "right/proper" prefix + established बोध (enlightenment) and संकल्प (resolve); not in MD-Mapping under this compound, compositional</t>
+          <t>Reused from KD 1 (see निवृत्ति-area rows below and KD-3 glossary); KD 2 explicitly glosses it as "बौद्धिक, सामाजिक एवं प्राकृतिक" (intellectual, social, and natural), confirming the KD 1 gloss</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>सद्विवेक</t>
+          <t>जागृति-त्रय, शक्ति-त्रय</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>sad-vivek</t>
+          <t>jagriti-traya, shakti-traya</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>right-wisdom</t>
+          <t>the "triad of awakening", the "triad of powers"</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>KD 2 p.46: सत् (right) + विवेक (wisdom); not in MD-Mapping, compositional, parallel to सम्यक्-बोध</t>
+          <t>KD 2: new parallel formations on the established "-त्रय = triad of X" pattern (see नियम-त्रय, व्यवहार-त्रय, अन्वेषण-त्रय, KD 1 glossary row). जागृति-त्रय = awakening of इच्छा/क्रिया/ज्ञान शक्ति (desire-, activity-, and knowledge-power); शक्ति-त्रय = the same three powers named directly</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>साध्य, साधक, साधन (उपासना में)</t>
+          <t>इच्छा शक्ति, क्रिया शक्ति, ज्ञान शक्ति</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>sadhya, sadhak, sadhan</t>
+          <t>ichha shakti, kriya shakti, gyan shakti</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>the aim, the seeker, the means</t>
+          <t>desire-power, activity-power, knowledge-power</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Reused from KD 3.17 (see row above) — KD 2 p.38 requires the same triad to remain integrated within upasana for it to succeed</t>
+          <t>KD 2: classical triad (kriya-shakti/iccha-shakti/jnana-shakti); not in MD-Mapping under this grouping, compositional</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>मत, सम्प्रदाय, वर्ग</t>
+          <t>ता-त्रय</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>mat, sampradaya, varga</t>
+          <t>tā-traya</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>creed, sect, class</t>
+          <t>the "triad of *-tā*"</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>KD 2 p.38: "मानव के स्वधर्म में ही मत, सम्प्रदाय, वर्ग तिरोहित हो जाते हैं" — not in MD-Mapping under this triad, compositional</t>
+          <t>KD 2 p.44: "स्वयं का मूल्यांकन 'ता-त्रय' की सीमा में होता है" (self-evaluation occurs within the domain of the tā-traya). UNCERTAIN — not in MD-Mapping; the surrounding text repeatedly pairs क्षमता/योग्यता/पात्रता (capacity/competence/worthiness), which is the likeliest referent, but the source does not gloss the compound explicitly here. Left transliterated and flagged for human review rather than asserted</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>वर्ग-भावना</t>
+          <t>अनुक्षण-विक्षण-वृत्ति, सहजावृत्ति</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>varga-bhavana</t>
+          <t>anukshan-vikshan-vritti, sahajavritti</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>class-sentiment</t>
+          <t>the moment-to-moment unbroken tendency; natural-recurrence</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>KD 2 p.35: not in MD-Mapping, compositional (वर्ग = class/group + भावना = sentiment)</t>
+          <t>KD 2 p.43/45: defined in-text as "the disappearance of moment-to-moment mediating obstruction." Not in MD-Mapping; compositional, glossed in-text on first use</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>सर्वमंगल, मांगल्य</t>
+          <t>तदाकार</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>sarva mangal, mangalya</t>
+          <t>tadakar</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>universal welfare, welfare</t>
+          <t>taking-the-form-of</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>KD 2: सर्व मंगल (universal welfare) is the shared aim underlying all upasanas; मांगल्य is its abstract-noun cognate. Not in MD-Mapping, compositional</t>
+          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>अभ्युदय</t>
+          <t>सम्यक्-बोध, सम्यक् संकल्प</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>abhyudaya</t>
+          <t>samyak-bodh, samyak sankalp</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>comprehensive resolution</t>
+          <t>right-enlightenment, right resolve</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
+          <t>KD 2: सम्यक् = classical "right/proper" prefix + established बोध (enlightenment) and संकल्प (resolve); not in MD-Mapping under this compound, compositional</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>न्यूनातिरेक</t>
+          <t>सद्विवेक</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>nyoonatirek</t>
+          <t>sad-vivek</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>deficiency-or-excess</t>
+          <t>right-wisdom</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>KD 2 p.44: न्यून (deficient) + अतिरेक (excess); describes faulty (imposed) self-evaluation. Not in MD-Mapping, compositional</t>
+          <t>KD 2 p.46: सत् (right) + विवेक (wisdom); not in MD-Mapping, compositional, parallel to सम्यक्-बोध</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>प्रभुसत्ता</t>
+          <t>साध्य, साधक, साधन (उपासना में)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>prabhusatta</t>
+          <t>sadhya, sadhak, sadhan</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>sovereignty</t>
+          <t>the aim, the seeker, the means</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
+          <t>Reused from KD 3.17 (see row above) — KD 2 p.38 requires the same triad to remain integrated within upasana for it to succeed</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>साम्राज्य</t>
+          <t>मत, सम्प्रदाय, वर्ग</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>samrajya</t>
+          <t>mat, sampradaya, varga</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>dominion</t>
+          <t>creed, sect, class</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>KD 2 p.48: kept as "dominion" rather than "sovereignty" specifically to avoid collision with प्रभुसत्ता above — both appear in this chapter as distinct stages in a causal chain</t>
+          <t>KD 2 p.38: "मानव के स्वधर्म में ही मत, सम्प्रदाय, वर्ग तिरोहित हो जाते हैं" — not in MD-Mapping under this triad, compositional</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>मानवेतर प्राणी</t>
+          <t>वर्ग-भावना</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>manavetar prani</t>
+          <t>varga-bhavana</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>beings other than human</t>
+          <t>class-sentiment</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>KD 2 p.48: parallel to the already-established मानवेत्तर प्रकृति = "nature-other-than-human" (KD 3.7 glossary row)</t>
+          <t>KD 2 p.35: not in MD-Mapping, compositional (वर्ग = class/group + भावना = sentiment)</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>विराग, वैराग्य</t>
+          <t>सर्वमंगल, मांगल्य</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>virag, vairagya</t>
+          <t>sarva mangal, mangalya</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>dispassion</t>
+          <t>universal welfare, welfare</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+          <t>KD 2: सर्व मंगल (universal welfare) is the shared aim underlying all upasanas; मांगल्य is its abstract-noun cognate. Not in MD-Mapping, compositional</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>आत्म-दीपन</t>
+          <t>अभ्युदय</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>atma-deepan</t>
+          <t>abhyudaya</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>self-illumination</t>
+          <t>comprehensive resolution</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>KD 2 p.48: दीपन = illumination/kindling; not in MD-Mapping, compositional, part of the आत्म-बोध → आत्म-दीपन → आत्म-विश्वास → ... causal chain</t>
+          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>पाण्डित्य</t>
+          <t>न्यूनातिरेक</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>panditya</t>
+          <t>nyoonatirek</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>scholarliness</t>
+          <t>deficiency-or-excess</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Per MD-Mapping; first appearance in the KD corpus at KD 2 p.31 ("परिमार्जनशीलता ही निपुणता एवं कुशलता, पाण्डित्य है")</t>
+          <t>KD 2 p.44: न्यून (deficient) + अतिरेक (excess); describes faulty (imposed) self-evaluation. Not in MD-Mapping, compositional</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>कासा, आकूति, मेधा (क्रिया/इच्छा/ज्ञान शक्ति के रूप में)</t>
+          <t>प्रभुसत्ता</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>kāsā, ākūti, medhā</t>
+          <t>prabhusatta</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>activity-power (kāsā), desire-power (ākūti), knowledge-power (medhā)</t>
+          <t>sovereignty</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Reused from KD 1 (glossary row above) — KD 2 p.47 re-invokes the same triad, now explicitly mapped onto क्रिया/इच्छा/ज्ञान शक्ति</t>
+          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
+          <t>साम्राज्य</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>samrajya</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>dominion</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>KD 2 p.48: kept as "dominion" rather than "sovereignty" specifically to avoid collision with प्रभुसत्ता above — both appear in this chapter as distinct stages in a causal chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>मानवेतर प्राणी</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>manavetar prani</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>beings other than human</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>KD 2 p.48: parallel to the already-established मानवेत्तर प्रकृति = "nature-other-than-human" (KD 3.7 glossary row)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>विराग, वैराग्य</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>virag, vairagya</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>dispassion</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>आत्म-दीपन</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>atma-deepan</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>self-illumination</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>KD 2 p.48: दीपन = illumination/kindling; not in MD-Mapping, compositional, part of the आत्म-बोध → आत्म-दीपन → आत्म-विश्वास → ... causal chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>पाण्डित्य</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>panditya</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>scholarliness</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Per MD-Mapping; first appearance in the KD corpus at KD 2 p.31 ("परिमार्जनशीलता ही निपुणता एवं कुशलता, पाण्डित्य है")</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>कासा, आकूति, मेधा (क्रिया/इच्छा/ज्ञान शक्ति के रूप में)</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>kāsā, ākūti, medhā</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>activity-power (kāsā), desire-power (ākūti), knowledge-power (medhā)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Reused from KD 1 (glossary row above) — KD 2 p.47 re-invokes the same triad, now explicitly mapped onto क्रिया/इच्छा/ज्ञान शक्ति</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
           <t>अवकाश</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B154" t="inlineStr">
         <is>
           <t>avakash</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C154" t="inlineStr">
         <is>
           <t>opportunity</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="D154" t="inlineStr">
         <is>
           <t>Settled per Raghava (2026-07-09): **not** "leisure." KD 1 p.14 (PDF p.39) glosses अवकाश (सम्भावना) → "opportunity (possibility)"; body/mind/wealth as means is itself opportunity; paired with अवसर ("occasion") in "necessity, occasion, and opportunity." Distinct from MD-Mapping's आकाश, अवकाश = "void" (space sense). MVD renders अवकाश एवम् अवसर as "opportunity and scope"</t>
         </is>
@@ -61470,10 +61602,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="114" min="1" max="1"/>
+    <col width="22" customWidth="1" style="114" min="1" max="1"/>
     <col width="58" customWidth="1" style="114" min="2" max="2"/>
     <col width="60" customWidth="1" style="114" min="3" max="3"/>
     <col width="60" customWidth="1" style="114" min="4" max="4"/>
@@ -61724,122 +61856,122 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>विस्तार</t>
+          <t>चुंबकीय बल सम्पन्नता</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>expanse</t>
+          <t>magnetic force-fullness</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>extension (span)</t>
+          <t>magnetic-force-full / magnetic force-fullness</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KD 3.14: "whatever length, breadth, and height a composition is spread over"; distinct from the compound विस्तार आयाम \= area</t>
+          <t>Per MD-Mapping चुंबकीय बल सम्पन्नता = magnetic force-fullness. Supersedes earlier "endowed with magnetic force" / "magnetic-force endowment". Retroactively corrected corpus-wide 2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>फलन</t>
+          <t>विस्तार</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>function/outcome</t>
+          <t>expanse</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>fruition</t>
+          <t>extension (span)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KD 3.15: evaluation on the basis of activity and fruition</t>
+          <t>KD 3.14: "whatever length, breadth, and height a composition is spread over"; distinct from the compound विस्तार आयाम \= area</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>नित्य वर्तमान</t>
+          <t>फलन</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eternal presence</t>
+          <t>function/outcome</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ever-present</t>
+          <t>fruition</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Settled per Raghava (July 2026); KD 3.15 predicate of kaal</t>
+          <t>KD 3.15: evaluation on the basis of activity and fruition</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>मेधस</t>
+          <t>नित्य वर्तमान</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>brain</t>
+          <t>eternal presence</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>brain / medhas</t>
+          <t>ever-present</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MD-Mapping: brain; KD 3.3 "medhas composition"</t>
+          <t>Settled per Raghava (July 2026); KD 3.15 predicate of kaal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>आत्मा</t>
+          <t>मेधस</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>atma</t>
+          <t>brain</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>left transliterated (atma, buddhi, chitta, vritti, mun/"mind")</t>
+          <t>brain / medhas</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KD 3.6: the five jeevan faculties (pūrvānukram), each carrying one of the five *sthiti* (state) activities — anubhav/atma (realisation), bodh/buddhi (enlightenment), chintan/chitta (contemplation), tulan/vritti (comparison), aswadan/mun (tasting) — and one of the five *gati* (motion) activities — praman/atma (evidence), ṛtambharā/buddhi (resoluteness), ichha/chitta (desire), vishleshan/vritti (analysis), chayan/mun (selection). MD-Mapping leaves all five untranslated; matches its own note under अंतर्नियामन ("पूर्वानुक्रम = वरीयता क्रम याने आत्मा, बुद्धि, चित्त, वृत्ति, मन")</t>
+          <t>MD-Mapping: brain; KD 3.3 "medhas composition"</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>बुद्धि</t>
+          <t>आत्मा</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>buddhi</t>
+          <t>atma</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61856,12 +61988,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>चित्त</t>
+          <t>बुद्धि</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>chitta</t>
+          <t>buddhi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61878,12 +62010,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>वृत्ति</t>
+          <t>चित्त</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>vritti</t>
+          <t>chitta</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -61900,12 +62032,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>मन</t>
+          <t>वृत्ति</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>mun</t>
+          <t>vritti</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61922,122 +62054,122 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>गठनपूर्णता</t>
+          <t>मन</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>constitutional completeness</t>
+          <t>mun</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>constitutional completeness, activity-completeness, conduct-completeness</t>
+          <t>left transliterated (atma, buddhi, chitta, vritti, mun/"mind")</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KD 3.3/3.4: the atom's three stages of development. गठनपूर्णता = "constitutional completeness" per MD-Mapping; क्रियापूर्णता and आचरणपूर्णता are parallel KD coinages (not in MD-Mapping), rendered analogously</t>
+          <t>KD 3.6: the five jeevan faculties (pūrvānukram), each carrying one of the five *sthiti* (state) activities — anubhav/atma (realisation), bodh/buddhi (enlightenment), chintan/chitta (contemplation), tulan/vritti (comparison), aswadan/mun (tasting) — and one of the five *gati* (motion) activities — praman/atma (evidence), ṛtambharā/buddhi (resoluteness), ichha/chitta (desire), vishleshan/vritti (analysis), chayan/mun (selection). MD-Mapping leaves all five untranslated; matches its own note under अंतर्नियामन ("पूर्वानुक्रम = वरीयता क्रम याने आत्मा, बुद्धि, चित्त, वृत्ति, मन")</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>यथास्थिति</t>
+          <t>गठनपूर्णता</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>existent state</t>
+          <t>constitutional completeness</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>actual condition</t>
+          <t>constitutional completeness, activity-completeness, conduct-completeness</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KD 3.4/3.5: distinct from अस्तित्व (existence) — the concrete, as-is condition of a thing/person, not "status quo" in the political sense</t>
+          <t>KD 3.3/3.4: the atom's three stages of development. गठनपूर्णता = "constitutional completeness" per MD-Mapping; क्रियापूर्णता and आचरणपूर्णता are parallel KD coinages (not in MD-Mapping), rendered analogously</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>तृप्ति</t>
+          <t>यथास्थिति</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Satisfaction</t>
+          <t>existent state</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>satiation</t>
+          <t>actual condition</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KD 3.6: jeevan's fulfilment through realisation (*anubhav*), recognised in human tradition as happiness, peace, and contentment</t>
+          <t>KD 3.4/3.5: distinct from अस्तित्व (existence) — the concrete, as-is condition of a thing/person, not "status quo" in the political sense</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>गुण</t>
+          <t>तृप्ति</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>properties</t>
+          <t>Satisfaction</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>satiation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08): "property," NOT "quality." MD-Mapping carries both readings (गुण = "properties" as a noun; गुण = "qualitative" as an adjective) — for KD's recurring रूप/गुण/स्वभाव/धर्म (form/property/essential nature/dharma) list of the four orders' predominant traits, and for chapter 3.10's title, गुण is a noun and takes "property." Retroactively corrected in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12, and KD-Karm-Darshan-English.md §3.13–3.15 (previously translated "quality") on 2026-07-08. Exception: the adjectival compound गुणात्मक परिवर्तन keeps MD-Mapping's own established "qualitative change/transformation" (KD 3.9) — "property-al" does not read in English, and MD-Mapping treats this compound as a separate row from bare गुण</t>
+          <t>KD 3.6: jeevan's fulfilment through realisation (*anubhav*), recognised in human tradition as happiness, peace, and contentment</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>सम</t>
+          <t>गुण</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>generative</t>
+          <t>properties</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>generative, degenerative, mediating</t>
+          <t>property</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
+          <t>Settled per Raghava (2026-07-08): "property," NOT "quality." MD-Mapping carries both readings (गुण = "properties" as a noun; गुण = "qualitative" as an adjective) — for KD's recurring रूप/गुण/स्वभाव/धर्म (form/property/essential nature/dharma) list of the four orders' predominant traits, and for chapter 3.10's title, गुण is a noun and takes "property." Retroactively corrected in KD-Karm-Darshan-English.md §3.4–3.6, KD-Karm-Darshan-English.md §3.11–3.12, and KD-Karm-Darshan-English.md §3.13–3.15 (previously translated "quality") on 2026-07-08. Exception: the adjectival compound गुणात्मक परिवर्तन keeps MD-Mapping's own established "qualitative change/transformation" (KD 3.9) — "property-al" does not read in English, and MD-Mapping treats this compound as a separate row from bare गुण</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>विषम</t>
+          <t>सम</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>degenerative</t>
+          <t>generative</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -62054,34 +62186,34 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>सारक</t>
+          <t>विषम</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Vitalising</t>
+          <t>degenerative</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>essential(ity), destructive(ness)</t>
+          <t>generative, degenerative, mediating</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KD 3.10: the two modes of स्वभाव (essential nature) in the prana state — sarakta = being abundant in itself and useful to the animal order; marakta = obstructing one's own seed-abundance and being disease/death-causing to the animal order</t>
+          <t>Per MD-Mapping (सम=generative, विषम=degenerative) and MVD running prose ("generative, degenerative, and mediative"). **Do not leave bare सम/विषम transliterated in analytical prose** — use generative / degenerative (MVD spelling: "degenerative", not "de-generative"). Optional (*sam*) / (*visham*) gloss only on first compound use if helpful (e.g. generative-degenerative (*sam-visham*)). Retroactively corrected in KD 1 (pp. 15–16, 25) on 2026-07-10 where *sam*/*visham* had been left italic-transliterated. मध्यस्थ here is an adjective describing the property that maintains a composition once formed ("mediating" in KD; MVD often "mediative"), distinct from मध्यस्थीयकरण (mediation, KD 3.11)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>मारक</t>
+          <t>सारक</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Devitalising</t>
+          <t>Vitalising</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -62098,56 +62230,56 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>पात्रता</t>
+          <t>मारक</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>receptivity</t>
+          <t>Devitalising</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>worthiness</t>
+          <t>essential(ity), destructive(ness)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
+          <t>KD 3.10: the two modes of स्वभाव (essential nature) in the prana state — sarakta = being abundant in itself and useful to the animal order; marakta = obstructing one's own seed-abundance and being disease/death-causing to the animal order</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>देव मानव</t>
+          <t>पात्रता</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>deific human</t>
+          <t>receptivity</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>god-human, divine human</t>
+          <t>worthiness</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>KD 3.10: literal rendering, judgment call; not in MD-Mapping</t>
+          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>दिव्य मानव</t>
+          <t>देव मानव</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>divine human</t>
+          <t>deific human</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -62164,34 +62296,34 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>पशु मानव</t>
+          <t>दिव्य मानव</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>animalistic human</t>
+          <t>divine human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>the animalistic human, the demonic human</t>
+          <t>god-human, divine human</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("animalistic human," "demonic human"). Retroactively corrected in KD-Karm-Darshan-English.md §3.9–3.10 on 2026-07-08 (previously "animal-human"/"demon-human") to match MD-Mapping exactly and align with KD 1's usage of the same pair</t>
+          <t>KD 3.10: literal rendering, judgment call; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>राक्षस मानव</t>
+          <t>पशु मानव</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>demonic human</t>
+          <t>animalistic human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -62208,34 +62340,34 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>दृष्टा</t>
+          <t>राक्षस मानव</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Seer</t>
+          <t>demonic human</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>seer, knower, known</t>
+          <t>the animalistic human, the demonic human</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Per MD-Mapping: दृष्टा=Seer, ज्ञाता=knower (not in PS), ज्ञेय=knowable (not in PS). KD 3.16-3.18 titles this triad "known" rather than MD-Mapping's literal "knowable" — reads more naturally as the object-pole of ज्ञान/ज्ञाता (knowledge/knower), a judgment call</t>
+          <t>Per MD-Mapping ("animalistic human," "demonic human"). Retroactively corrected in KD-Karm-Darshan-English.md §3.9–3.10 on 2026-07-08 (previously "animal-human"/"demon-human") to match MD-Mapping exactly and align with KD 1's usage of the same pair</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ज्ञाता</t>
+          <t>दृष्टा</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>knower</t>
+          <t>Seer</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -62252,12 +62384,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ज्ञेय</t>
+          <t>ज्ञाता</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>knowable</t>
+          <t>knower</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -62274,56 +62406,56 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>भोक्ता</t>
+          <t>ज्ञेय</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>enjoyer, experiencer</t>
+          <t>knowable</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>doer, enjoyer</t>
+          <t>seer, knower, known</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Compositional; कर्त्ता=doer (agent), भोक्ता=enjoyer (experiencer of result). KD 3.18 title</t>
+          <t>Per MD-Mapping: दृष्टा=Seer, ज्ञाता=knower (not in PS), ज्ञेय=knowable (not in PS). KD 3.16-3.18 titles this triad "known" rather than MD-Mapping's literal "knowable" — reads more naturally as the object-pole of ज्ञान/ज्ञाता (knowledge/knower), a judgment call</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>दृश्य</t>
+          <t>भोक्ता</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>scene</t>
+          <t>enjoyer, experiencer</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>the seeing, the seen, seeing/philosophy</t>
+          <t>doer, enjoyer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>KD 3.17: the seer-triad parallel to ज्ञान/ज्ञाता/ज्ञेय; left transliterated with bracketed gloss on first use, not in MD-Mapping under these exact senses</t>
+          <t>Compositional; कर्त्ता=doer (agent), भोक्ता=enjoyer (experiencer of result). KD 3.18 title</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>दर्शन</t>
+          <t>दृश्य</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Holistic view, Worldview, Philosophy</t>
+          <t>scene</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -62340,34 +62472,34 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ध्यान</t>
+          <t>दर्शन</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>concentration</t>
+          <t>Holistic view, Worldview, Philosophy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>attention, attender, object of attention</t>
+          <t>the seeing, the seen, seeing/philosophy</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>KD 3.17: not in MD-Mapping under this triad; compositional, parallel structure to ज्ञान/ज्ञाता/ज्ञेय</t>
+          <t>KD 3.17: the seer-triad parallel to ज्ञान/ज्ञाता/ज्ञेय; left transliterated with bracketed gloss on first use, not in MD-Mapping under these exact senses</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ध्याता</t>
+          <t>ध्यान</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>the one who concentrates</t>
+          <t>concentration</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -62384,12 +62516,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ध्येय</t>
+          <t>ध्याता</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>object of concentration</t>
+          <t>the one who concentrates</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -62406,34 +62538,34 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>साध्य</t>
+          <t>ध्येय</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>aim</t>
+          <t>object of concentration</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>aim, seeker, means</t>
+          <t>attention, attender, object of attention</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Per MD-Mapping: साध्य=aim, साधक=the seeker, साधन=the means. KD 3.17 triad</t>
+          <t>KD 3.17: not in MD-Mapping under this triad; compositional, parallel structure to ज्ञान/ज्ञाता/ज्ञेय</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>साधक</t>
+          <t>साध्य</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>the seeker</t>
+          <t>aim</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -62450,12 +62582,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>साधन</t>
+          <t>साधक</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>the means</t>
+          <t>the seeker</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -62472,34 +62604,34 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>अध्यात्मवाद</t>
+          <t>साधन</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>spiritualism, adhyatma-vada</t>
+          <t>the means</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>spiritualism, god-centred-ism, materialism-of-the-beyond</t>
+          <t>aim, seeker, means</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (kept close to transliteration: adhyatma-vada, Adhidaivika-vada, adhi-bhautikvad); KD 3.17 names the three classical schools collectively subsumed under आदर्शवाद (idealism)</t>
+          <t>Per MD-Mapping: साध्य=aim, साधक=the seeker, साधन=the means. KD 3.17 triad</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>अधिदैवीवाद</t>
+          <t>अध्यात्मवाद</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Adhidaivika-vada</t>
+          <t>spiritualism, adhyatma-vada</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -62516,12 +62648,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>अधिभौतिकवाद</t>
+          <t>अधिदैवीवाद</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>adhi-bhautikvad</t>
+          <t>Adhidaivika-vada</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -62538,78 +62670,78 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>संचेतना</t>
+          <t>अधिभौतिकवाद</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>consciousness, human consciousness, humane consciousness</t>
+          <t>adhi-bhautikvad</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>awareness</t>
+          <t>spiritualism, god-centred-ism, materialism-of-the-beyond</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), OVERRIDING MD-Mapping/SB's "Humane Consciousness" (SB Ch7 title) — "awareness" avoids collision with चेतना/जीव चेतना ("consciousness," e.g. "animal consciousness," KD 1) and चैतन्य ("conscious," e.g. "conscious activity," "material-conscious nature"), which stay untouched. Applies to संचेतनशील too ("awareness-endowed"). **Audit rule (2026-07-08 remediation):** grep for "human consciousness" / "higher-human consciousness" — replace with awareness / higher-awareness wherever the Hindi source is संचेतना; keep "consciousness" only for चेतना (e.g. "social consciousness" = सामाजिक चेतना, "consciousness-development" = चेतना विकास)</t>
+          <t>Per MD-Mapping (kept close to transliteration: adhyatma-vada, Adhidaivika-vada, adhi-bhautikvad); KD 3.17 names the three classical schools collectively subsumed under आदर्शवाद (idealism)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>अभीष्ट</t>
+          <t>संचेतना</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Aim</t>
+          <t>consciousness, human consciousness, humane consciousness</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>desire</t>
+          <t>awareness</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "desideratum" (itself an override of MD-Mapping's "Aim," chosen to avoid colliding with साध्य=aim). Note: this reintroduces a collision with इच्छा (the general term for desire throughout KD) — अभीष्ट and इच्छा are now both "desire" in English; distinguish by context if needed (अभीष्ट is the wished-for/happiness-directed sense, इच्छा the general faculty/act of desiring). साध्य keeps "aim." Where the source explicitly glosses one with the other ("साध्य (अभीष्ट)"), rendered as "the aim (the desire)"</t>
+          <t>Settled per Raghava (2026-07-08), OVERRIDING MD-Mapping/SB's "Humane Consciousness" (SB Ch7 title) — "awareness" avoids collision with चेतना/जीव चेतना ("consciousness," e.g. "animal consciousness," KD 1) and चैतन्य ("conscious," e.g. "conscious activity," "material-conscious nature"), which stay untouched. Applies to संचेतनशील too ("awareness-endowed"). **Audit rule (2026-07-08 remediation):** grep for "human consciousness" / "higher-human consciousness" — replace with awareness / higher-awareness wherever the Hindi source is संचेतना; keep "consciousness" only for चेतना (e.g. "social consciousness" = सामाजिक चेतना, "consciousness-development" = चेतना विकास)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>कृत</t>
+          <t>अभीष्ट</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>Aim</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>done, caused, intended</t>
+          <t>desire</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "done, caused-to-be-done, and approved"/"consented-to." MD-Mapping's कृत="doing," कारित="getting done," अनुमोदित="consenting" — kept close but simplified; अनुमोदित specifically rendered "intended" rather than "approved"/"consenting" per this decision. Retrofitted in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances, including the related noun अनुमोदन→"intention") and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance) on 2026-07-08</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "desideratum" (itself an override of MD-Mapping's "Aim," chosen to avoid colliding with साध्य=aim). Note: this reintroduces a collision with इच्छा (the general term for desire throughout KD) — अभीष्ट and इच्छा are now both "desire" in English; distinguish by context if needed (अभीष्ट is the wished-for/happiness-directed sense, इच्छा the general faculty/act of desiring). साध्य keeps "aim." Where the source explicitly glosses one with the other ("साध्य (अभीष्ट)"), rendered as "the aim (the desire)"</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>कारित</t>
+          <t>कृत</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>getting done</t>
+          <t>doing</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -62626,12 +62758,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>अनुमोदित</t>
+          <t>कारित</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>consenting</t>
+          <t>getting done</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -62648,276 +62780,276 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>फल</t>
+          <t>अनुमोदित</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>consequence</t>
+          <t>consenting</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>done, caused, intended</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "fruit" — "phal means result of the action (karma)." Retrofitted in KD-Karm-Darshan-English.md on 2026-07-08 wherever फल stood alone (not फलन=fruition, not a फल-परिणाम compound, not literal fruit as food). See परिणाम for the resolved collision and the फल-परिणाम compound convention</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "done, caused-to-be-done, and approved"/"consented-to." MD-Mapping's कृत="doing," कारित="getting done," अनुमोदित="consenting" — kept close but simplified; अनुमोदित specifically rendered "intended" rather than "approved"/"consenting" per this decision. Retrofitted in KD-Karm-Darshan-English.md §3.11–3.12 (3 instances, including the related noun अनुमोदन→"intention") and KD-Karm-Darshan-English.md §3.16–3.18 (1 instance) on 2026-07-08</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>अनुभूति</t>
+          <t>फल</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>realisation</t>
+          <t>consequence</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>experiencing</t>
+          <t>result</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Judgment call, OVERRIDING MD-Mapping's "realisation" — MD-Mapping gives both अनुभूति and अनुभव as "realisation," but अनुभव is deeply entrenched across chapter 3 in KD-Karm-Darshan-English.md as "realisation" and the two words appear together/nearby throughout KD 1 (e.g. "सत्यानुभूति," "अनुभूति आनन्द"). अनुभव keeps "realisation"; अनुभूति becomes "experiencing" (the felt/sensed process) to keep them distinguishable</t>
+          <t>Settled per Raghava (2026-07-08), superseding this project's earlier "fruit" — "phal means result of the action (karma)." Retrofitted in KD-Karm-Darshan-English.md on 2026-07-08 wherever फल stood alone (not फलन=fruition, not a फल-परिणाम compound, not literal fruit as food). See परिणाम for the resolved collision and the फल-परिणाम compound convention</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>संस्कार</t>
+          <t>अनुभूति</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sanskar</t>
+          <t>realisation</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>*sanskar* (left transliterated)</t>
+          <t>experiencing</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Per MD-Mapping (kept as "Sanskar," not translated). Settled per this project (2026-07-08): KD 1 uses संस्कार and संस्कृति together constantly (e.g. "संस्कार, संस्कृति व सभ्यता") — collapsing both to "culture" erases the distinction. संस्कार = the individual's cultural conditioning/refinement (kept as *sanskar*); संस्कृति = the collective/civilizational achievement (kept as "culture"); सभ्यता = "civilisation"</t>
+          <t>Judgment call, OVERRIDING MD-Mapping's "realisation" — MD-Mapping gives both अनुभूति and अनुभव as "realisation," but अनुभव is deeply entrenched across chapter 3 in KD-Karm-Darshan-English.md as "realisation" and the two words appear together/nearby throughout KD 1 (e.g. "सत्यानुभूति," "अनुभूति आनन्द"). अनुभव keeps "realisation"; अनुभूति becomes "experiencing" (the felt/sensed process) to keep them distinguishable</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>सभ्यता</t>
+          <t>संस्कार</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>civilization, civility</t>
+          <t>Sanskar</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>civilisation</t>
+          <t>*sanskar* (left transliterated)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("civilization, civility")</t>
+          <t>Per MD-Mapping (kept as "Sanskar," not translated). Settled per this project (2026-07-08): KD 1 uses संस्कार and संस्कृति together constantly (e.g. "संस्कार, संस्कृति व सभ्यता") — collapsing both to "culture" erases the distinction. संस्कार = the individual's cultural conditioning/refinement (kept as *sanskar*); संस्कृति = the collective/civilizational achievement (kept as "culture"); सभ्यता = "civilisation"</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>काम</t>
+          <t>सभ्यता</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>lust</t>
+          <t>civilization, civility</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>*kama* (desire)</t>
+          <t>civilisation</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>KD 1: contextual exception — MD-Mapping's "lust" is too narrow for the classical चतुर्वर्ग (मोक्ष/धर्म/काम/अर्थ) listing, where काम denotes desire/pleasure as a life-aim, not specifically sexual desire. Left transliterated with gloss "(desire)" on first use, distinct from इच्छा (the general term for desire throughout KD)</t>
+          <t>Per MD-Mapping ("civilization, civility")</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>अर्थ</t>
+          <t>काम</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>resources</t>
+          <t>lust</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>wealth (contextual)</t>
+          <t>*kama* (desire)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("resources"), rendered "wealth" for readability in the चतुर्वर्ग list and wealth/resource contexts ("अर्थ तन, मन, धन है"). CONTEXTUAL EXCEPTION: where अर्थ is used epistemically (e.g. "सम्पूर्ण अर्थ का पूर्ण अर्थ अनुभव ही है"), it means "meaning," not "wealth" — judge from context</t>
+          <t>KD 1: contextual exception — MD-Mapping's "lust" is too narrow for the classical चतुर्वर्ग (मोक्ष/धर्म/काम/अर्थ) listing, where काम denotes desire/pleasure as a life-aim, not specifically sexual desire. Left transliterated with gloss "(desire)" on first use, distinct from इच्छा (the general term for desire throughout KD)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>मेधा</t>
+          <t>अर्थ</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>intellect</t>
+          <t>resources</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>left transliterated</t>
+          <t>wealth (contextual)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>KD 1: an obscure classical triad of "union-born intellect" (योग-जन्य-बुद्धि), not in MD-Mapping. Glossed in-text on first occurrence (poet/sage-artist; divine worker; divine knower with complete knowledge) — judgment call, flag for review against a Sanskrit dictionary if precision matters</t>
+          <t>Per MD-Mapping ("resources"), rendered "wealth" for readability in the चतुर्वर्ग list and wealth/resource contexts ("अर्थ तन, मन, धन है"). CONTEXTUAL EXCEPTION: where अर्थ is used epistemically (e.g. "सम्पूर्ण अर्थ का पूर्ण अर्थ अनुभव ही है"), it means "meaning," not "wealth" — judge from context</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>निवृत्ति</t>
+          <t>मेधा</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Disencumberance, Disinclination</t>
+          <t>intellect</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>disencumberance</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
+          <t>KD 1: an obscure classical triad of "union-born intellect" (योग-जन्य-बुद्धि), not in MD-Mapping. Glossed in-text on first occurrence (poet/sage-artist; divine worker; divine knower with complete knowledge) — judgment call, flag for review against a Sanskrit dictionary if precision matters</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>निवृत्ति</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>cause</t>
+          <t>Disencumberance, Disinclination</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>gross, subtle, causal</t>
+          <t>disencumberance</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
+          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>उपासना</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>worship, upasana</t>
+          <t>cause</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Upasana (worship)</t>
+          <t>gross, subtle, causal</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
+          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>नश्वरत्व</t>
+          <t>उपासना</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>mortality</t>
+          <t>worship, upasana</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>perishability</t>
+          <t>Upasana (worship)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
+          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>देवात्मा</t>
+          <t>नश्वरत्व</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>deific-self</t>
+          <t>mortality</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>the deific soul, the elemental soul, the divine soul</t>
+          <t>perishability</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>दिव्यात्मा</t>
+          <t>देवात्मा</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>divine-self</t>
+          <t>deific-self</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -62934,130 +63066,152 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>विद्या</t>
+          <t>दिव्यात्मा</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>divine-self</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>learning, sub-learning, base learning</t>
+          <t>the deific soul, the elemental soul, the divine soul</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
+          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>तदाकार</t>
+          <t>विद्या</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>absolute-resonance</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>taking-the-form-of</t>
+          <t>learning, sub-learning, base learning</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
+          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>अभ्युदय</t>
+          <t>तदाकार</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>comprehensive resolution (Abhyudaya)</t>
+          <t>absolute-resonance</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>comprehensive resolution</t>
+          <t>taking-the-form-of</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
+          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>प्रभुसत्ता</t>
+          <t>अभ्युदय</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Supreme order</t>
+          <t>comprehensive resolution (Abhyudaya)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>sovereignty</t>
+          <t>comprehensive resolution</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
+          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>वैराग्य</t>
+          <t>प्रभुसत्ता</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>detachment</t>
+          <t>Supreme order</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>dispassion</t>
+          <t>sovereignty</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>वैराग्य</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>detachment</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>dispassion</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>अवकाश</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>void</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>opportunity</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Settled per Raghava (2026-07-09): **not** "leisure." KD 1 p.14 (PDF p.39) glosses अवकाश (सम्भावना) → "opportunity (possibility)"; body/mind/wealth as means is itself opportunity; paired with अवसर ("occasion") in "necessity, occasion, and opportunity." Distinct from MD-Mapping's आकाश, अवकाश = "void" (space sense). MVD renders अवकाश एवम् अवसर as "opportunity and scope"</t>
         </is>

</xml_diff>

<commit_message>
Expand MD-Mapping from MVD/SB (Phase 4) and add KD verification.
Add 60 curated glossary rows from freq>=2 pair evidence, ship candidate/evidence/review-card tooling, and report KD glossary overrides vs the updated mapping.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
+++ b/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
@@ -960,7 +960,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2147"/>
+  <dimension ref="A1:K2207"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.44" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="23.22" customWidth="1" style="114" min="1" max="1"/>
@@ -58177,6 +58177,1626 @@
       <c r="I2147" s="0" t="inlineStr">
         <is>
           <t>SB p.15; SB p.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" s="0" t="inlineStr">
+        <is>
+          <t>अखण्ड</t>
+        </is>
+      </c>
+      <c r="B2148" s="0" t="inlineStr">
+        <is>
+          <t>undivided</t>
+        </is>
+      </c>
+      <c r="C2148" s="0" t="inlineStr">
+        <is>
+          <t>akhand</t>
+        </is>
+      </c>
+      <c r="F2148" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अखण्ड सामाजिकता / अखण्ड समाज = undivided sociality / undivided society (MVD).</t>
+        </is>
+      </c>
+      <c r="I2148" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" s="0" t="inlineStr">
+        <is>
+          <t>पूरक</t>
+        </is>
+      </c>
+      <c r="B2149" s="0" t="inlineStr">
+        <is>
+          <t>complementary</t>
+        </is>
+      </c>
+      <c r="C2149" s="0" t="inlineStr">
+        <is>
+          <t>purak</t>
+        </is>
+      </c>
+      <c r="F2149" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: एकसूत्रता = being helpful and complementary for mutual awakening.</t>
+        </is>
+      </c>
+      <c r="I2149" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.102</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" s="0" t="inlineStr">
+        <is>
+          <t>जंगल युग</t>
+        </is>
+      </c>
+      <c r="B2150" s="0" t="inlineStr">
+        <is>
+          <t>Jungle Age</t>
+        </is>
+      </c>
+      <c r="C2150" s="0" t="inlineStr">
+        <is>
+          <t>jangal yug</t>
+        </is>
+      </c>
+      <c r="F2150" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: SB periodization Jungle Age → Stone Age → Iron Age → Submission Age → Struggle Age.</t>
+        </is>
+      </c>
+      <c r="I2150" s="0" t="inlineStr">
+        <is>
+          <t>SB p.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" s="0" t="inlineStr">
+        <is>
+          <t>भाषा</t>
+        </is>
+      </c>
+      <c r="B2151" s="0" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="C2151" s="0" t="inlineStr">
+        <is>
+          <t>bhasha</t>
+        </is>
+      </c>
+      <c r="F2151" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: व्यवहार, भाव व भाषा = behaviour, sentiments, and language.</t>
+        </is>
+      </c>
+      <c r="I2151" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.229</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" s="0" t="inlineStr">
+        <is>
+          <t>अवसर</t>
+        </is>
+      </c>
+      <c r="B2152" s="0" t="inlineStr">
+        <is>
+          <t>opportunity / opportunism (contextual)</t>
+        </is>
+      </c>
+      <c r="C2152" s="0" t="inlineStr">
+        <is>
+          <t>avsar</t>
+        </is>
+      </c>
+      <c r="F2152" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: bare अवसर often 'opportunity'; in न्याय तथा अवसर भेद paired with opportunism (cf. अवसरवादी).</t>
+        </is>
+      </c>
+      <c r="I2152" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.213</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" s="0" t="inlineStr">
+        <is>
+          <t>वर्ग</t>
+        </is>
+      </c>
+      <c r="B2153" s="0" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C2153" s="0" t="inlineStr">
+        <is>
+          <t>varg</t>
+        </is>
+      </c>
+      <c r="F2153" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: जाति, वर्ग, मत, सम्प्रदाय = castes, classes, beliefs, and sects.</t>
+        </is>
+      </c>
+      <c r="I2153" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.267</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" s="0" t="inlineStr">
+        <is>
+          <t>विपरीत</t>
+        </is>
+      </c>
+      <c r="B2154" s="0" t="inlineStr">
+        <is>
+          <t>opposite / contrary</t>
+        </is>
+      </c>
+      <c r="C2154" s="0" t="inlineStr">
+        <is>
+          <t>viparit</t>
+        </is>
+      </c>
+      <c r="F2154" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: इसके विपरीत = in contrast / opposite (e.g. दया vs द्वेष).</t>
+        </is>
+      </c>
+      <c r="I2154" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.189</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" s="0" t="inlineStr">
+        <is>
+          <t>अल्प चेतन</t>
+        </is>
+      </c>
+      <c r="B2155" s="0" t="inlineStr">
+        <is>
+          <t>partially conscious / partially awakened</t>
+        </is>
+      </c>
+      <c r="C2155" s="0" t="inlineStr">
+        <is>
+          <t>alp chetan</t>
+        </is>
+      </c>
+      <c r="F2155" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अल्प चेतन in the fivefold consciousness scale = partially conscious / partially awakened.</t>
+        </is>
+      </c>
+      <c r="I2155" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.274</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" s="0" t="inlineStr">
+        <is>
+          <t>अविकसित</t>
+        </is>
+      </c>
+      <c r="B2156" s="0" t="inlineStr">
+        <is>
+          <t>undeveloped</t>
+        </is>
+      </c>
+      <c r="C2156" s="0" t="inlineStr">
+        <is>
+          <t>aviksit</t>
+        </is>
+      </c>
+      <c r="F2156" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अविकसित इकाई = undeveloped unit (contrast विकसित).</t>
+        </is>
+      </c>
+      <c r="I2156" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.290</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" s="0" t="inlineStr">
+        <is>
+          <t>बन्धन</t>
+        </is>
+      </c>
+      <c r="B2157" s="0" t="inlineStr">
+        <is>
+          <t>bondage</t>
+        </is>
+      </c>
+      <c r="C2157" s="0" t="inlineStr">
+        <is>
+          <t>bandhan</t>
+        </is>
+      </c>
+      <c r="F2157" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: mirage and delusion which is bondage.</t>
+        </is>
+      </c>
+      <c r="I2157" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.140</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" s="0" t="inlineStr">
+        <is>
+          <t>मार्ग</t>
+        </is>
+      </c>
+      <c r="B2158" s="0" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="C2158" s="0" t="inlineStr">
+        <is>
+          <t>marg</t>
+        </is>
+      </c>
+      <c r="F2158" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: मार्ग प्रशस्त = pave the path (moral policy).</t>
+        </is>
+      </c>
+      <c r="I2158" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.243</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" s="0" t="inlineStr">
+        <is>
+          <t>श्रेष्ठ</t>
+        </is>
+      </c>
+      <c r="B2159" s="0" t="inlineStr">
+        <is>
+          <t>superior</t>
+        </is>
+      </c>
+      <c r="C2159" s="0" t="inlineStr">
+        <is>
+          <t>shreshth</t>
+        </is>
+      </c>
+      <c r="F2159" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: स्व… को श्रेष्ठ तथा अन्य को नेष्ट = one's own as superior, others as inferior (conceit).</t>
+        </is>
+      </c>
+      <c r="I2159" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.185</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" s="0" t="inlineStr">
+        <is>
+          <t>समर्थन</t>
+        </is>
+      </c>
+      <c r="B2160" s="0" t="inlineStr">
+        <is>
+          <t>endorsement / support</t>
+        </is>
+      </c>
+      <c r="C2160" s="0" t="inlineStr">
+        <is>
+          <t>samarthan</t>
+        </is>
+      </c>
+      <c r="F2160" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: समर्थन व पालन = endorsing and adhering.</t>
+        </is>
+      </c>
+      <c r="I2160" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.257</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" s="0" t="inlineStr">
+        <is>
+          <t>सर्वमानव</t>
+        </is>
+      </c>
+      <c r="B2161" s="0" t="inlineStr">
+        <is>
+          <t>all humans</t>
+        </is>
+      </c>
+      <c r="C2161" s="0" t="inlineStr">
+        <is>
+          <t>sarvamanav</t>
+        </is>
+      </c>
+      <c r="F2161" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: सर्वमानव में, से, के लिए = in, by, and for all humans.</t>
+        </is>
+      </c>
+      <c r="I2161" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.300</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" s="0" t="inlineStr">
+        <is>
+          <t>अर्ध चेतन</t>
+        </is>
+      </c>
+      <c r="B2162" s="0" t="inlineStr">
+        <is>
+          <t>half-conscious / half-awakened</t>
+        </is>
+      </c>
+      <c r="C2162" s="0" t="inlineStr">
+        <is>
+          <t>ardh chetan</t>
+        </is>
+      </c>
+      <c r="F2162" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अर्ध चेतन in the fivefold consciousness scale.</t>
+        </is>
+      </c>
+      <c r="I2162" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.274</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" s="0" t="inlineStr">
+        <is>
+          <t>द्योतक</t>
+        </is>
+      </c>
+      <c r="B2163" s="0" t="inlineStr">
+        <is>
+          <t>indicative</t>
+        </is>
+      </c>
+      <c r="C2163" s="0" t="inlineStr">
+        <is>
+          <t>dyotak</t>
+        </is>
+      </c>
+      <c r="F2163" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: मानवीयता का द्योतक = indicative of humaneness.</t>
+        </is>
+      </c>
+      <c r="I2163" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.176</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" s="0" t="inlineStr">
+        <is>
+          <t>नस्ल</t>
+        </is>
+      </c>
+      <c r="B2164" s="0" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C2164" s="0" t="inlineStr">
+        <is>
+          <t>nasl</t>
+        </is>
+      </c>
+      <c r="F2164" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: रंग और नस्ल = colour and race (SB).</t>
+        </is>
+      </c>
+      <c r="I2164" s="0" t="inlineStr">
+        <is>
+          <t>SB p.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" s="0" t="inlineStr">
+        <is>
+          <t>माता-पिता</t>
+        </is>
+      </c>
+      <c r="B2165" s="0" t="inlineStr">
+        <is>
+          <t>mother-father / parents</t>
+        </is>
+      </c>
+      <c r="C2165" s="0" t="inlineStr">
+        <is>
+          <t>mata-pita</t>
+        </is>
+      </c>
+      <c r="F2165" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: one of the defined family relationships; life of a parent.</t>
+        </is>
+      </c>
+      <c r="I2165" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.257</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" s="0" t="inlineStr">
+        <is>
+          <t>पिता</t>
+        </is>
+      </c>
+      <c r="B2166" s="0" t="inlineStr">
+        <is>
+          <t>father / parent</t>
+        </is>
+      </c>
+      <c r="C2166" s="0" t="inlineStr">
+        <is>
+          <t>pita</t>
+        </is>
+      </c>
+      <c r="F2166" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: see माता-पिता row; parental relationship definition.</t>
+        </is>
+      </c>
+      <c r="I2166" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.257</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" s="0" t="inlineStr">
+        <is>
+          <t>मौलिक</t>
+        </is>
+      </c>
+      <c r="B2167" s="0" t="inlineStr">
+        <is>
+          <t>fundamental</t>
+        </is>
+      </c>
+      <c r="C2167" s="0" t="inlineStr">
+        <is>
+          <t>maulik</t>
+        </is>
+      </c>
+      <c r="F2167" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: मौलिक मूल्य = fundamental value (gratitude).</t>
+        </is>
+      </c>
+      <c r="I2167" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" s="0" t="inlineStr">
+        <is>
+          <t>संभावना</t>
+        </is>
+      </c>
+      <c r="B2168" s="0" t="inlineStr">
+        <is>
+          <t>possibility</t>
+        </is>
+      </c>
+      <c r="C2168" s="0" t="inlineStr">
+        <is>
+          <t>sambhavna</t>
+        </is>
+      </c>
+      <c r="F2168" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: तृप्ति की संभावना = possibility of satisfaction.</t>
+        </is>
+      </c>
+      <c r="I2168" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.166</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" s="0" t="inlineStr">
+        <is>
+          <t>दिशा</t>
+        </is>
+      </c>
+      <c r="B2169" s="0" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="C2169" s="0" t="inlineStr">
+        <is>
+          <t>disha</t>
+        </is>
+      </c>
+      <c r="F2169" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: दिशा निर्धारण = determining the direction (science/vigyan).</t>
+        </is>
+      </c>
+      <c r="I2169" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.170</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" s="0" t="inlineStr">
+        <is>
+          <t>भूमि</t>
+        </is>
+      </c>
+      <c r="B2170" s="0" t="inlineStr">
+        <is>
+          <t>Earth / land</t>
+        </is>
+      </c>
+      <c r="C2170" s="0" t="inlineStr">
+        <is>
+          <t>bhumi</t>
+        </is>
+      </c>
+      <c r="F2170" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: भूमि स्वर्ग हो = May the Earth be heavenly.</t>
+        </is>
+      </c>
+      <c r="I2170" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" s="0" t="inlineStr">
+        <is>
+          <t>पालन</t>
+        </is>
+      </c>
+      <c r="B2171" s="0" t="inlineStr">
+        <is>
+          <t>adherence / observance</t>
+        </is>
+      </c>
+      <c r="C2171" s="0" t="inlineStr">
+        <is>
+          <t>palan</t>
+        </is>
+      </c>
+      <c r="F2171" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: समर्थन व पालन = endorsing and adhering.</t>
+        </is>
+      </c>
+      <c r="I2171" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.257</t>
+        </is>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" s="0" t="inlineStr">
+        <is>
+          <t>आधारित</t>
+        </is>
+      </c>
+      <c r="B2172" s="0" t="inlineStr">
+        <is>
+          <t>based on</t>
+        </is>
+      </c>
+      <c r="C2172" s="0" t="inlineStr">
+        <is>
+          <t>adharit</t>
+        </is>
+      </c>
+      <c r="F2172" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: श्रम मूल्य… आधारित = based on evaluation and exchange of labour.</t>
+        </is>
+      </c>
+      <c r="I2172" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.269</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" s="0" t="inlineStr">
+        <is>
+          <t>समुदाय, समुदायों</t>
+        </is>
+      </c>
+      <c r="B2173" s="0" t="inlineStr">
+        <is>
+          <t>community / communities</t>
+        </is>
+      </c>
+      <c r="C2173" s="0" t="inlineStr">
+        <is>
+          <t>samuday</t>
+        </is>
+      </c>
+      <c r="F2173" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: human communities formed around freedom from fear.</t>
+        </is>
+      </c>
+      <c r="I2173" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" s="0" t="inlineStr">
+        <is>
+          <t>अमानवीय दृष्टि</t>
+        </is>
+      </c>
+      <c r="B2174" s="0" t="inlineStr">
+        <is>
+          <t>inhumane perspective</t>
+        </is>
+      </c>
+      <c r="C2174" s="0" t="inlineStr">
+        <is>
+          <t>amanviya drishti</t>
+        </is>
+      </c>
+      <c r="F2174" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: explicit MVD gloss Inhumane Perspective (amanveeya drishti).</t>
+        </is>
+      </c>
+      <c r="I2174" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" s="0" t="inlineStr">
+        <is>
+          <t>असंतुलन</t>
+        </is>
+      </c>
+      <c r="B2175" s="0" t="inlineStr">
+        <is>
+          <t>imbalance / disparity</t>
+        </is>
+      </c>
+      <c r="C2175" s="0" t="inlineStr">
+        <is>
+          <t>asantulan</t>
+        </is>
+      </c>
+      <c r="F2175" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अमीरी-गरीबी का असंतुलन = disparity between rich and poor.</t>
+        </is>
+      </c>
+      <c r="I2175" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.267</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" s="0" t="inlineStr">
+        <is>
+          <t>आर्थिक सुरक्षा</t>
+        </is>
+      </c>
+      <c r="B2176" s="0" t="inlineStr">
+        <is>
+          <t>economic security</t>
+        </is>
+      </c>
+      <c r="C2176" s="0" t="inlineStr">
+        <is>
+          <t>arthik suraksha</t>
+        </is>
+      </c>
+      <c r="F2176" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: explicit MVD heading Economic Security.</t>
+        </is>
+      </c>
+      <c r="I2176" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.265</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" s="0" t="inlineStr">
+        <is>
+          <t>इकाईयाँ</t>
+        </is>
+      </c>
+      <c r="B2177" s="0" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="C2177" s="0" t="inlineStr">
+        <is>
+          <t>ikaiyan</t>
+        </is>
+      </c>
+      <c r="F2177" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: इकाईयाँ अनंत = units are countless.</t>
+        </is>
+      </c>
+      <c r="I2177" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" s="0" t="inlineStr">
+        <is>
+          <t>नियंत्रित, नियन्त्रण</t>
+        </is>
+      </c>
+      <c r="B2178" s="0" t="inlineStr">
+        <is>
+          <t>regulated / regulation</t>
+        </is>
+      </c>
+      <c r="C2178" s="0" t="inlineStr">
+        <is>
+          <t>niyantrit</t>
+        </is>
+      </c>
+      <c r="F2178" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: प्रकृति नियंत्रित एवं संरक्षित = nature regulated and conserved; नियन्त्रण = regulation of prana.</t>
+        </is>
+      </c>
+      <c r="I2178" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" s="0" t="inlineStr">
+        <is>
+          <t>पृथ्वी</t>
+        </is>
+      </c>
+      <c r="B2179" s="0" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="C2179" s="0" t="inlineStr">
+        <is>
+          <t>prithvi</t>
+        </is>
+      </c>
+      <c r="F2179" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: Geography is study of the Earth's structure.</t>
+        </is>
+      </c>
+      <c r="I2179" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.136</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" s="0" t="inlineStr">
+        <is>
+          <t>शाकाहारी</t>
+        </is>
+      </c>
+      <c r="B2180" s="0" t="inlineStr">
+        <is>
+          <t>herbivorous</t>
+        </is>
+      </c>
+      <c r="C2180" s="0" t="inlineStr">
+        <is>
+          <t>shakahari</t>
+        </is>
+      </c>
+      <c r="F2180" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: शाकाहारी और मांसाहारी = herbivorous and carnivorous.</t>
+        </is>
+      </c>
+      <c r="I2180" s="0" t="inlineStr">
+        <is>
+          <t>SB p.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" s="0" t="inlineStr">
+        <is>
+          <t>मांसाहारी</t>
+        </is>
+      </c>
+      <c r="B2181" s="0" t="inlineStr">
+        <is>
+          <t>carnivorous</t>
+        </is>
+      </c>
+      <c r="C2181" s="0" t="inlineStr">
+        <is>
+          <t>mansahari</t>
+        </is>
+      </c>
+      <c r="F2181" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: paired with शाकाहारी in SB animal-order discussion.</t>
+        </is>
+      </c>
+      <c r="I2181" s="0" t="inlineStr">
+        <is>
+          <t>SB p.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" s="0" t="inlineStr">
+        <is>
+          <t>सम्पर्क</t>
+        </is>
+      </c>
+      <c r="B2182" s="0" t="inlineStr">
+        <is>
+          <t>association / contact</t>
+        </is>
+      </c>
+      <c r="C2182" s="0" t="inlineStr">
+        <is>
+          <t>sampark</t>
+        </is>
+      </c>
+      <c r="F2182" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: सम्पर्क एवं संबंध = associations and relationships (paired with संबंध).</t>
+        </is>
+      </c>
+      <c r="I2182" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.242</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" s="0" t="inlineStr">
+        <is>
+          <t>स्वर्ग</t>
+        </is>
+      </c>
+      <c r="B2183" s="0" t="inlineStr">
+        <is>
+          <t>heaven / heavenly</t>
+        </is>
+      </c>
+      <c r="C2183" s="0" t="inlineStr">
+        <is>
+          <t>svarg</t>
+        </is>
+      </c>
+      <c r="F2183" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: भूमि स्वर्ग हो = May the Earth be heavenly.</t>
+        </is>
+      </c>
+      <c r="I2183" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" s="0" t="inlineStr">
+        <is>
+          <t>अधिकतम</t>
+        </is>
+      </c>
+      <c r="B2184" s="0" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="C2184" s="0" t="inlineStr">
+        <is>
+          <t>adhiktam</t>
+        </is>
+      </c>
+      <c r="F2184" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: अधिकतम श्रम = maximum effort.</t>
+        </is>
+      </c>
+      <c r="I2184" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.266</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" s="0" t="inlineStr">
+        <is>
+          <t>निरन्तरता</t>
+        </is>
+      </c>
+      <c r="B2185" s="0" t="inlineStr">
+        <is>
+          <t>continuity</t>
+        </is>
+      </c>
+      <c r="C2185" s="0" t="inlineStr">
+        <is>
+          <t>nirantarta</t>
+        </is>
+      </c>
+      <c r="F2185" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: कृतज्ञता की निरन्तरता = continuity of gratitude.</t>
+        </is>
+      </c>
+      <c r="I2185" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" s="0" t="inlineStr">
+        <is>
+          <t>स्व पुरुष</t>
+        </is>
+      </c>
+      <c r="B2186" s="0" t="inlineStr">
+        <is>
+          <t>one's husband / marital faithfulness (contextual)</t>
+        </is>
+      </c>
+      <c r="C2186" s="0" t="inlineStr">
+        <is>
+          <t>sva purush</t>
+        </is>
+      </c>
+      <c r="F2186" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: स्वनारी/स्व पुरुष in the righteous-wealth / marital-faithfulness policy triad.</t>
+        </is>
+      </c>
+      <c r="I2186" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.267</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" s="0" t="inlineStr">
+        <is>
+          <t>प्रवृत्ति, प्रवृत्तियाँ</t>
+        </is>
+      </c>
+      <c r="B2187" s="0" t="inlineStr">
+        <is>
+          <t>tendency / tendencies</t>
+        </is>
+      </c>
+      <c r="C2187" s="0" t="inlineStr">
+        <is>
+          <t>pravritti</t>
+        </is>
+      </c>
+      <c r="F2187" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: विचार व प्रवृत्तियाँ = thoughts and tendencies.</t>
+        </is>
+      </c>
+      <c r="I2187" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.211</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" s="0" t="inlineStr">
+        <is>
+          <t>प्रसन्नता</t>
+        </is>
+      </c>
+      <c r="B2188" s="0" t="inlineStr">
+        <is>
+          <t>happiness / gladly</t>
+        </is>
+      </c>
+      <c r="C2188" s="0" t="inlineStr">
+        <is>
+          <t>prasannata</t>
+        </is>
+      </c>
+      <c r="F2188" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: प्रसन्नता पूर्वक = happily (generosity definition).</t>
+        </is>
+      </c>
+      <c r="I2188" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.52</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" s="0" t="inlineStr">
+        <is>
+          <t>मनुष्य</t>
+        </is>
+      </c>
+      <c r="B2189" s="0" t="inlineStr">
+        <is>
+          <t>human / humans</t>
+        </is>
+      </c>
+      <c r="C2189" s="0" t="inlineStr">
+        <is>
+          <t>manushya</t>
+        </is>
+      </c>
+      <c r="F2189" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: मनुष्य देवता हो = May humans be deities.</t>
+        </is>
+      </c>
+      <c r="I2189" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" s="0" t="inlineStr">
+        <is>
+          <t>वर्ग विहीन</t>
+        </is>
+      </c>
+      <c r="B2190" s="0" t="inlineStr">
+        <is>
+          <t>classless</t>
+        </is>
+      </c>
+      <c r="C2190" s="0" t="inlineStr">
+        <is>
+          <t>varg vihin</t>
+        </is>
+      </c>
+      <c r="F2190" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: वर्ग विहीन समाज = classless society.</t>
+        </is>
+      </c>
+      <c r="I2190" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" s="0" t="inlineStr">
+        <is>
+          <t>वैयक्तिक</t>
+        </is>
+      </c>
+      <c r="B2191" s="0" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="C2191" s="0" t="inlineStr">
+        <is>
+          <t>vaiyaktik</t>
+        </is>
+      </c>
+      <c r="F2191" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: वैयक्तिक जीवन व जीविका = individual life and livelihood.</t>
+        </is>
+      </c>
+      <c r="I2191" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.168</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" s="0" t="inlineStr">
+        <is>
+          <t>संरक्षित</t>
+        </is>
+      </c>
+      <c r="B2192" s="0" t="inlineStr">
+        <is>
+          <t>protected / conserved</t>
+        </is>
+      </c>
+      <c r="C2192" s="0" t="inlineStr">
+        <is>
+          <t>sanrakshit</t>
+        </is>
+      </c>
+      <c r="F2192" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: नियंत्रित तथा संरक्षित = regulated and protected/conserved.</t>
+        </is>
+      </c>
+      <c r="I2192" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.144</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" s="0" t="inlineStr">
+        <is>
+          <t>योग्य</t>
+        </is>
+      </c>
+      <c r="B2193" s="0" t="inlineStr">
+        <is>
+          <t>fit / worthy / suitable</t>
+        </is>
+      </c>
+      <c r="C2193" s="0" t="inlineStr">
+        <is>
+          <t>yogya</t>
+        </is>
+      </c>
+      <c r="F2193" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: योगानुभूति योग्य विकास = development fit for realisation of yog; distinct from योग्यता (ability).</t>
+        </is>
+      </c>
+      <c r="I2193" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.165</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" s="0" t="inlineStr">
+        <is>
+          <t>सुलभ</t>
+        </is>
+      </c>
+      <c r="B2194" s="0" t="inlineStr">
+        <is>
+          <t>accessible</t>
+        </is>
+      </c>
+      <c r="C2194" s="0" t="inlineStr">
+        <is>
+          <t>sulabh</t>
+        </is>
+      </c>
+      <c r="F2194" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: समाधान व समझ सुलभ = resolution and understanding become accessible.</t>
+        </is>
+      </c>
+      <c r="I2194" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.290</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" s="0" t="inlineStr">
+        <is>
+          <t>संभव</t>
+        </is>
+      </c>
+      <c r="B2195" s="0" t="inlineStr">
+        <is>
+          <t>possible</t>
+        </is>
+      </c>
+      <c r="C2195" s="0" t="inlineStr">
+        <is>
+          <t>sambhav</t>
+        </is>
+      </c>
+      <c r="F2195" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: …से ही संभव है = is possible only through…</t>
+        </is>
+      </c>
+      <c r="I2195" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.172</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" s="0" t="inlineStr">
+        <is>
+          <t>स्थान</t>
+        </is>
+      </c>
+      <c r="B2196" s="0" t="inlineStr">
+        <is>
+          <t>place / position</t>
+        </is>
+      </c>
+      <c r="C2196" s="0" t="inlineStr">
+        <is>
+          <t>sthan</t>
+        </is>
+      </c>
+      <c r="F2196" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: महत्वपूर्ण स्थान = significant position/place.</t>
+        </is>
+      </c>
+      <c r="I2196" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.192</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" s="0" t="inlineStr">
+        <is>
+          <t>स्वरुप, स्वरूप</t>
+        </is>
+      </c>
+      <c r="B2197" s="0" t="inlineStr">
+        <is>
+          <t>form / aspect</t>
+        </is>
+      </c>
+      <c r="C2197" s="0" t="inlineStr">
+        <is>
+          <t>svarup</t>
+        </is>
+      </c>
+      <c r="F2197" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: तीन स्वरुप में = under three headings/forms (theism categories).</t>
+        </is>
+      </c>
+      <c r="I2197" s="0" t="inlineStr">
+        <is>
+          <t>SB p.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" s="0" t="inlineStr">
+        <is>
+          <t>नारी</t>
+        </is>
+      </c>
+      <c r="B2198" s="0" t="inlineStr">
+        <is>
+          <t>woman / wife (contextual)</t>
+        </is>
+      </c>
+      <c r="C2198" s="0" t="inlineStr">
+        <is>
+          <t>nari</t>
+        </is>
+      </c>
+      <c r="F2198" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: स्व-नारी/पर-नारी in marital faithfulness vs adultery discussion.</t>
+        </is>
+      </c>
+      <c r="I2198" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.189</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" s="0" t="inlineStr">
+        <is>
+          <t>इंगित</t>
+        </is>
+      </c>
+      <c r="B2199" s="0" t="inlineStr">
+        <is>
+          <t>indicated / signalled</t>
+        </is>
+      </c>
+      <c r="C2199" s="0" t="inlineStr">
+        <is>
+          <t>ingit</t>
+        </is>
+      </c>
+      <c r="F2199" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: इंगित होने वाले सम्पूर्ण संकेतों = all the signals indicated/received.</t>
+        </is>
+      </c>
+      <c r="I2199" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.345</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" s="0" t="inlineStr">
+        <is>
+          <t>उपलब्ध</t>
+        </is>
+      </c>
+      <c r="B2200" s="0" t="inlineStr">
+        <is>
+          <t>available / allocated</t>
+        </is>
+      </c>
+      <c r="C2200" s="0" t="inlineStr">
+        <is>
+          <t>upalabdh</t>
+        </is>
+      </c>
+      <c r="F2200" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: साधन उपलब्ध कराना = allocating/making resources available.</t>
+        </is>
+      </c>
+      <c r="I2200" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.268</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" s="0" t="inlineStr">
+        <is>
+          <t>वृत्ति, वृति</t>
+        </is>
+      </c>
+      <c r="B2201" s="0" t="inlineStr">
+        <is>
+          <t>vritti</t>
+        </is>
+      </c>
+      <c r="C2201" s="0" t="inlineStr">
+        <is>
+          <t>vritti</t>
+        </is>
+      </c>
+      <c r="F2201" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: kept as vritti in MVD English (mun → vritti → chitta → buddhi hierarchy).</t>
+        </is>
+      </c>
+      <c r="I2201" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.286</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" s="0" t="inlineStr">
+        <is>
+          <t>संदर्भ</t>
+        </is>
+      </c>
+      <c r="B2202" s="0" t="inlineStr">
+        <is>
+          <t>context / respect (with respect to)</t>
+        </is>
+      </c>
+      <c r="C2202" s="0" t="inlineStr">
+        <is>
+          <t>sandarbh</t>
+        </is>
+      </c>
+      <c r="F2202" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: मानव के संदर्भ में = with respect to humans.</t>
+        </is>
+      </c>
+      <c r="I2202" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.231</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" s="0" t="inlineStr">
+        <is>
+          <t>क्षतिग्रस्त</t>
+        </is>
+      </c>
+      <c r="B2203" s="0" t="inlineStr">
+        <is>
+          <t>damaged / destroyed</t>
+        </is>
+      </c>
+      <c r="C2203" s="0" t="inlineStr">
+        <is>
+          <t>kshatigrast</t>
+        </is>
+      </c>
+      <c r="F2203" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: सर्वाधिक क्षतिग्रस्त = maximum destruction/damage to nature.</t>
+        </is>
+      </c>
+      <c r="I2203" s="0" t="inlineStr">
+        <is>
+          <t>SB p.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" s="0" t="inlineStr">
+        <is>
+          <t>रहस्यमय</t>
+        </is>
+      </c>
+      <c r="B2204" s="0" t="inlineStr">
+        <is>
+          <t>mysterious</t>
+        </is>
+      </c>
+      <c r="C2204" s="0" t="inlineStr">
+        <is>
+          <t>rahasyamay</t>
+        </is>
+      </c>
+      <c r="F2204" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: रहस्यमय लगता है = may seem mysterious.</t>
+        </is>
+      </c>
+      <c r="I2204" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.295</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" s="0" t="inlineStr">
+        <is>
+          <t>समाहित</t>
+        </is>
+      </c>
+      <c r="B2205" s="0" t="inlineStr">
+        <is>
+          <t>encompassed / included</t>
+        </is>
+      </c>
+      <c r="C2205" s="0" t="inlineStr">
+        <is>
+          <t>samahit</t>
+        </is>
+      </c>
+      <c r="F2205" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: व्यापक में समाहित = encompassed within omnipresence.</t>
+        </is>
+      </c>
+      <c r="I2205" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" s="0" t="inlineStr">
+        <is>
+          <t>स्वाभाविक</t>
+        </is>
+      </c>
+      <c r="B2206" s="0" t="inlineStr">
+        <is>
+          <t>natural / typically</t>
+        </is>
+      </c>
+      <c r="C2206" s="0" t="inlineStr">
+        <is>
+          <t>svabhavik</t>
+        </is>
+      </c>
+      <c r="F2206" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: typically/naturally occurs (brother-sister recognition).</t>
+        </is>
+      </c>
+      <c r="I2206" s="0" t="inlineStr">
+        <is>
+          <t>MVD p.250</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" s="0" t="inlineStr">
+        <is>
+          <t>धातु युग</t>
+        </is>
+      </c>
+      <c r="B2207" s="0" t="inlineStr">
+        <is>
+          <t>Iron Age</t>
+        </is>
+      </c>
+      <c r="C2207" s="0" t="inlineStr">
+        <is>
+          <t>dhatu yug</t>
+        </is>
+      </c>
+      <c r="F2207" s="0" t="inlineStr">
+        <is>
+          <t>Phase 4 curated: SB periodization Stone Age to Iron Age (धातु युग).</t>
+        </is>
+      </c>
+      <c r="I2207" s="0" t="inlineStr">
+        <is>
+          <t>SB p.23</t>
         </is>
       </c>
     </row>
@@ -61602,7 +63222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="114" min="1" max="1"/>
@@ -63132,86 +64752,108 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>अभ्युदय</t>
+          <t>वर्ग</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>comprehensive resolution (Abhyudaya)</t>
+          <t>class</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>comprehensive resolution</t>
+          <t>creed, sect, class</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
+          <t>KD 2 p.38: "मानव के स्वधर्म में ही मत, सम्प्रदाय, वर्ग तिरोहित हो जाते हैं" — not in MD-Mapping under this triad, compositional</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>प्रभुसत्ता</t>
+          <t>अभ्युदय</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Supreme order</t>
+          <t>comprehensive resolution (Abhyudaya)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>sovereignty</t>
+          <t>comprehensive resolution</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
+          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>वैराग्य</t>
+          <t>प्रभुसत्ता</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>detachment</t>
+          <t>Supreme order</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>dispassion</t>
+          <t>sovereignty</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>वैराग्य</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>detachment</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>dispassion</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>अवकाश</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>void</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>opportunity</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Settled per Raghava (2026-07-09): **not** "leisure." KD 1 p.14 (PDF p.39) glosses अवकाश (सम्भावना) → "opportunity (possibility)"; body/mind/wealth as means is itself opportunity; paired with अवसर ("occasion") in "necessity, occasion, and opportunity." Distinct from MD-Mapping's आकाश, अवकाश = "void" (space sense). MVD renders अवकाश एवम् अवसर as "opportunity and scope"</t>
         </is>

</xml_diff>

<commit_message>
Add 35 KD glossary terms to MD-Mapping and fix KD triad consistency.
Absorb formerly missing KD lemmas into MD-Mapping (rows 2208-2242), standardize the capacity/ability/receptivity triad and desires-trio wording, and regenerate KD PDFs/glossary.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
+++ b/References/Madhyasth-Darshan/KD-Karm-Darshan-English/KD-Translation-Glossary.xlsx
@@ -960,7 +960,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2207"/>
+  <dimension ref="A1:K2242"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.44" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="23.22" customWidth="1" style="114" min="1" max="1"/>
@@ -59797,6 +59797,951 @@
       <c r="I2207" s="0" t="inlineStr">
         <is>
           <t>SB p.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" s="0" t="inlineStr">
+        <is>
+          <t>मध्यांश</t>
+        </is>
+      </c>
+      <c r="B2208" s="0" t="inlineStr">
+        <is>
+          <t>nucleus</t>
+        </is>
+      </c>
+      <c r="C2208" s="0" t="inlineStr">
+        <is>
+          <t>madhyansh</t>
+        </is>
+      </c>
+      <c r="F2208" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.1/3.11 — central particle(s) of the atom. Settled per Raghava.</t>
+        </is>
+      </c>
+      <c r="I2208" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.1/3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" s="0" t="inlineStr">
+        <is>
+          <t>अच्छी दूरी</t>
+        </is>
+      </c>
+      <c r="B2209" s="0" t="inlineStr">
+        <is>
+          <t>good distance</t>
+        </is>
+      </c>
+      <c r="C2209" s="0" t="inlineStr">
+        <is>
+          <t>acchi doori</t>
+        </is>
+      </c>
+      <c r="F2209" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): equilibrium separation maintained by the nucleus / between bodies.</t>
+        </is>
+      </c>
+      <c r="I2209" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" s="0" t="inlineStr">
+        <is>
+          <t>मध्यस्थीयकरण</t>
+        </is>
+      </c>
+      <c r="B2210" s="0" t="inlineStr">
+        <is>
+          <t>mediation</t>
+        </is>
+      </c>
+      <c r="C2210" s="0" t="inlineStr">
+        <is>
+          <t>madhyasthiyakaran</t>
+        </is>
+      </c>
+      <c r="F2210" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.11 — what modern force/power studies are said to deny.</t>
+        </is>
+      </c>
+      <c r="I2210" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" s="0" t="inlineStr">
+        <is>
+          <t>चुम्बकीय धारा</t>
+        </is>
+      </c>
+      <c r="B2211" s="0" t="inlineStr">
+        <is>
+          <t>magnetic current</t>
+        </is>
+      </c>
+      <c r="C2211" s="0" t="inlineStr">
+        <is>
+          <t>chumbakiya dhara</t>
+        </is>
+      </c>
+      <c r="F2211" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.13 — electricity as flow from its fragmentation.</t>
+        </is>
+      </c>
+      <c r="I2211" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" s="0" t="inlineStr">
+        <is>
+          <t>विद्युतवाहिता</t>
+        </is>
+      </c>
+      <c r="B2212" s="0" t="inlineStr">
+        <is>
+          <t>electric conduction</t>
+        </is>
+      </c>
+      <c r="C2212" s="0" t="inlineStr">
+        <is>
+          <t>vidyutvahita</t>
+        </is>
+      </c>
+      <c r="F2212" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.13 — radio/TV waves as electricity-borne word/sound.</t>
+        </is>
+      </c>
+      <c r="I2212" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" s="0" t="inlineStr">
+        <is>
+          <t>संकोचन प्रसारण</t>
+        </is>
+      </c>
+      <c r="B2213" s="0" t="inlineStr">
+        <is>
+          <t>contraction-expansion</t>
+        </is>
+      </c>
+      <c r="C2213" s="0" t="inlineStr">
+        <is>
+          <t>sankochan prasaran</t>
+        </is>
+      </c>
+      <c r="F2213" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.13 — mechanism of flow/pressure in a medium.</t>
+        </is>
+      </c>
+      <c r="I2213" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" s="0" t="inlineStr">
+        <is>
+          <t>अण्डाकार</t>
+        </is>
+      </c>
+      <c r="B2214" s="0" t="inlineStr">
+        <is>
+          <t>elliptic</t>
+        </is>
+      </c>
+      <c r="C2214" s="0" t="inlineStr">
+        <is>
+          <t>andakar</t>
+        </is>
+      </c>
+      <c r="F2214" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7 — Earth's orbital path. Settled per Raghava.</t>
+        </is>
+      </c>
+      <c r="I2214" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" s="0" t="inlineStr">
+        <is>
+          <t>ससम्मुखता</t>
+        </is>
+      </c>
+      <c r="B2215" s="0" t="inlineStr">
+        <is>
+          <t>facing-ness</t>
+        </is>
+      </c>
+      <c r="C2215" s="0" t="inlineStr">
+        <is>
+          <t>sasammukhta</t>
+        </is>
+      </c>
+      <c r="F2215" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7 — Earth's face toward the Sun.</t>
+        </is>
+      </c>
+      <c r="I2215" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" s="0" t="inlineStr">
+        <is>
+          <t>सौर व्यूह</t>
+        </is>
+      </c>
+      <c r="B2216" s="0" t="inlineStr">
+        <is>
+          <t>solar system (solar array)</t>
+        </is>
+      </c>
+      <c r="C2216" s="0" t="inlineStr">
+        <is>
+          <t>saur vyuh</t>
+        </is>
+      </c>
+      <c r="F2216" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7/3.11.</t>
+        </is>
+      </c>
+      <c r="I2216" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7/3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" s="0" t="inlineStr">
+        <is>
+          <t>ग्रह-गोल</t>
+        </is>
+      </c>
+      <c r="B2217" s="0" t="inlineStr">
+        <is>
+          <t>planet-orb</t>
+        </is>
+      </c>
+      <c r="C2217" s="0" t="inlineStr">
+        <is>
+          <t>grah-gol</t>
+        </is>
+      </c>
+      <c r="F2217" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7.</t>
+        </is>
+      </c>
+      <c r="I2217" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" s="0" t="inlineStr">
+        <is>
+          <t>संक्रमणीयता</t>
+        </is>
+      </c>
+      <c r="B2218" s="0" t="inlineStr">
+        <is>
+          <t>transition-ness</t>
+        </is>
+      </c>
+      <c r="C2218" s="0" t="inlineStr">
+        <is>
+          <t>sankramaniyata</t>
+        </is>
+      </c>
+      <c r="F2218" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.3 abstract noun of संक्रमण (transition).</t>
+        </is>
+      </c>
+      <c r="I2218" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" s="0" t="inlineStr">
+        <is>
+          <t>विकिरणीयता</t>
+        </is>
+      </c>
+      <c r="B2219" s="0" t="inlineStr">
+        <is>
+          <t>radiativeness</t>
+        </is>
+      </c>
+      <c r="C2219" s="0" t="inlineStr">
+        <is>
+          <t>vikiraniyata</t>
+        </is>
+      </c>
+      <c r="F2219" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.3 — emission property of undigested atoms.</t>
+        </is>
+      </c>
+      <c r="I2219" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" s="0" t="inlineStr">
+        <is>
+          <t>विकिरणीय द्रव्य</t>
+        </is>
+      </c>
+      <c r="B2220" s="0" t="inlineStr">
+        <is>
+          <t>radiant (radioactive) materials</t>
+        </is>
+      </c>
+      <c r="C2220" s="0" t="inlineStr">
+        <is>
+          <t>vikiraniya dravya</t>
+        </is>
+      </c>
+      <c r="F2220" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.11.</t>
+        </is>
+      </c>
+      <c r="I2220" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" s="0" t="inlineStr">
+        <is>
+          <t>संतुलनीकरण</t>
+        </is>
+      </c>
+      <c r="B2221" s="0" t="inlineStr">
+        <is>
+          <t>equilibration</t>
+        </is>
+      </c>
+      <c r="C2221" s="0" t="inlineStr">
+        <is>
+          <t>santulanikaran</t>
+        </is>
+      </c>
+      <c r="F2221" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7.</t>
+        </is>
+      </c>
+      <c r="I2221" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" s="0" t="inlineStr">
+        <is>
+          <t>आवर्तनशीलता</t>
+        </is>
+      </c>
+      <c r="B2222" s="0" t="inlineStr">
+        <is>
+          <t>cyclicality</t>
+        </is>
+      </c>
+      <c r="C2222" s="0" t="inlineStr">
+        <is>
+          <t>avartansheelta</t>
+        </is>
+      </c>
+      <c r="F2222" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7/3.15 — water cycle; recurrence basis of time-reckoning.</t>
+        </is>
+      </c>
+      <c r="I2222" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7/3.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" s="0" t="inlineStr">
+        <is>
+          <t>तापोद्दीपन</t>
+        </is>
+      </c>
+      <c r="B2223" s="0" t="inlineStr">
+        <is>
+          <t>heat-stimulation</t>
+        </is>
+      </c>
+      <c r="C2223" s="0" t="inlineStr">
+        <is>
+          <t>tapoddipan</t>
+        </is>
+      </c>
+      <c r="F2223" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.7.</t>
+        </is>
+      </c>
+      <c r="I2223" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" s="0" t="inlineStr">
+        <is>
+          <t>समकेन्द्रीय रेखा</t>
+        </is>
+      </c>
+      <c r="B2224" s="0" t="inlineStr">
+        <is>
+          <t>concentric line</t>
+        </is>
+      </c>
+      <c r="C2224" s="0" t="inlineStr">
+        <is>
+          <t>samkendriya rekha</t>
+        </is>
+      </c>
+      <c r="F2224" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.14.</t>
+        </is>
+      </c>
+      <c r="I2224" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" s="0" t="inlineStr">
+        <is>
+          <t>घटी, पल</t>
+        </is>
+      </c>
+      <c r="B2225" s="0" t="inlineStr">
+        <is>
+          <t>ghati, pal (time units)</t>
+        </is>
+      </c>
+      <c r="C2225" s="0" t="inlineStr">
+        <is>
+          <t>ghati, pal</t>
+        </is>
+      </c>
+      <c r="F2225" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.15 — left transliterated as traditional time units.</t>
+        </is>
+      </c>
+      <c r="I2225" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" s="0" t="inlineStr">
+        <is>
+          <t>चिराकांक्षा, चिराकाँक्षा</t>
+        </is>
+      </c>
+      <c r="B2226" s="0" t="inlineStr">
+        <is>
+          <t>abiding aspiration</t>
+        </is>
+      </c>
+      <c r="C2226" s="0" t="inlineStr">
+        <is>
+          <t>chira-akanksha</t>
+        </is>
+      </c>
+      <c r="F2226" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.6 — चिर (lasting) + आकांक्षा (aspiration).</t>
+        </is>
+      </c>
+      <c r="I2226" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" s="0" t="inlineStr">
+        <is>
+          <t>सचेष्ट</t>
+        </is>
+      </c>
+      <c r="B2227" s="0" t="inlineStr">
+        <is>
+          <t>earnestly active</t>
+        </is>
+      </c>
+      <c r="C2227" s="0" t="inlineStr">
+        <is>
+          <t>sachesht</t>
+        </is>
+      </c>
+      <c r="F2227" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.6 — alert, diligent striving toward the human goal.</t>
+        </is>
+      </c>
+      <c r="I2227" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" s="0" t="inlineStr">
+        <is>
+          <t>ब्रह्मवाद, आत्मवाद, जातिवाद, नस्लवाद, वंशवाद</t>
+        </is>
+      </c>
+      <c r="B2228" s="0" t="inlineStr">
+        <is>
+          <t>Brahma-doctrine, self-doctrine, casteism, racism, lineage-ism</t>
+        </is>
+      </c>
+      <c r="C2228" s="0" t="inlineStr">
+        <is>
+          <t>brahmavad, atmavad, jativad, naslvad, vanshvad</t>
+        </is>
+      </c>
+      <c r="F2228" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.16 — compositional -वाद (doctrine/ism) compounds.</t>
+        </is>
+      </c>
+      <c r="I2228" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" s="0" t="inlineStr">
+        <is>
+          <t>उद्घाता</t>
+        </is>
+      </c>
+      <c r="B2229" s="0" t="inlineStr">
+        <is>
+          <t>herald</t>
+        </is>
+      </c>
+      <c r="C2229" s="0" t="inlineStr">
+        <is>
+          <t>udghata</t>
+        </is>
+      </c>
+      <c r="F2229" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.18 — human being as one who announces/evidences awakened status.</t>
+        </is>
+      </c>
+      <c r="I2229" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" s="0" t="inlineStr">
+        <is>
+          <t>औकात</t>
+        </is>
+      </c>
+      <c r="B2230" s="0" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="C2230" s="0" t="inlineStr">
+        <is>
+          <t>aukat</t>
+        </is>
+      </c>
+      <c r="F2230" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 3.16 — capacity/standing of human body-composition across generations.</t>
+        </is>
+      </c>
+      <c r="I2230" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 3.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" s="0" t="inlineStr">
+        <is>
+          <t>वेदना</t>
+        </is>
+      </c>
+      <c r="B2231" s="0" t="inlineStr">
+        <is>
+          <t>pain</t>
+        </is>
+      </c>
+      <c r="C2231" s="0" t="inlineStr">
+        <is>
+          <t>vedana</t>
+        </is>
+      </c>
+      <c r="F2231" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — pressure of accepting the unacceptable; distinct from संवेदना (sensation).</t>
+        </is>
+      </c>
+      <c r="I2231" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1; MVD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" s="0" t="inlineStr">
+        <is>
+          <t>मति, सुमति, अनुमति</t>
+        </is>
+      </c>
+      <c r="B2232" s="0" t="inlineStr">
+        <is>
+          <t>mati, sumati, anumati (left transliterated)</t>
+        </is>
+      </c>
+      <c r="C2232" s="0" t="inlineStr">
+        <is>
+          <t>mati, sumati, anumati</t>
+        </is>
+      </c>
+      <c r="F2232" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — triad of righteous-action-born intellect (सुकर्म-जन्य-बुद्धि); left transliterated.</t>
+        </is>
+      </c>
+      <c r="I2232" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" s="0" t="inlineStr">
+        <is>
+          <t>अमति, कुमति, दुर्मति</t>
+        </is>
+      </c>
+      <c r="B2233" s="0" t="inlineStr">
+        <is>
+          <t>amati, kumati, durmati (left transliterated)</t>
+        </is>
+      </c>
+      <c r="C2233" s="0" t="inlineStr">
+        <is>
+          <t>amati, kumati, durmati</t>
+        </is>
+      </c>
+      <c r="F2233" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — triad of unrighteous-action-born tendency; parallel to मति/सुमति/अनुमति.</t>
+        </is>
+      </c>
+      <c r="I2233" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" s="0" t="inlineStr">
+        <is>
+          <t>पुण्यात्मा, पापात्मा</t>
+        </is>
+      </c>
+      <c r="B2234" s="0" t="inlineStr">
+        <is>
+          <t>the meritorious soul, the sinful soul</t>
+        </is>
+      </c>
+      <c r="C2234" s="0" t="inlineStr">
+        <is>
+          <t>punyatma, papatma</t>
+        </is>
+      </c>
+      <c r="F2234" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — compositional pair with सुखी/दुखी across five states.</t>
+        </is>
+      </c>
+      <c r="I2234" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" s="0" t="inlineStr">
+        <is>
+          <t>रजोगुण, तमोगुण, सत्वगुण</t>
+        </is>
+      </c>
+      <c r="B2235" s="0" t="inlineStr">
+        <is>
+          <t>rajoguna, tamoguna, sattvaguna (left transliterated)</t>
+        </is>
+      </c>
+      <c r="C2235" s="0" t="inlineStr">
+        <is>
+          <t>rajoguna, tamoguna, sattvaguna</t>
+        </is>
+      </c>
+      <c r="F2235" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — classical three गुण; mapped onto sam/visham/mediating.</t>
+        </is>
+      </c>
+      <c r="I2235" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" s="0" t="inlineStr">
+        <is>
+          <t>मानवीयतापूर्ण (X), अतिमानवीयतापूर्ण (X)</t>
+        </is>
+      </c>
+      <c r="B2236" s="0" t="inlineStr">
+        <is>
+          <t>humane (X) / higher-humane (X)</t>
+        </is>
+      </c>
+      <c r="C2236" s="0" t="inlineStr">
+        <is>
+          <t>manviyatapurna, atimanviyatapurna</t>
+        </is>
+      </c>
+      <c r="F2236" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): pattern rule — X-पूर्ण as plain adjective (humane / higher-humane), not "X-replete-with-humaneness". Distinct from bare मानवीयता nouns and other -पूर्ण compounds.</t>
+        </is>
+      </c>
+      <c r="I2236" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; MVD p.3, p.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" s="0" t="inlineStr">
+        <is>
+          <t>गम्यता</t>
+        </is>
+      </c>
+      <c r="B2237" s="0" t="inlineStr">
+        <is>
+          <t>the destination</t>
+        </is>
+      </c>
+      <c r="C2237" s="0" t="inlineStr">
+        <is>
+          <t>gamyata</t>
+        </is>
+      </c>
+      <c r="F2237" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 1 — abstract noun of गम्य/गन्तव्य (destination).</t>
+        </is>
+      </c>
+      <c r="I2237" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" s="0" t="inlineStr">
+        <is>
+          <t>सद्विवेक</t>
+        </is>
+      </c>
+      <c r="B2238" s="0" t="inlineStr">
+        <is>
+          <t>right-wisdom</t>
+        </is>
+      </c>
+      <c r="C2238" s="0" t="inlineStr">
+        <is>
+          <t>sad-vivek</t>
+        </is>
+      </c>
+      <c r="F2238" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 2 — सत् + विवेक; parallel to सम्यक्-बोध.</t>
+        </is>
+      </c>
+      <c r="I2238" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" s="0" t="inlineStr">
+        <is>
+          <t>सर्वमंगल, मांगल्य</t>
+        </is>
+      </c>
+      <c r="B2239" s="0" t="inlineStr">
+        <is>
+          <t>universal welfare, welfare</t>
+        </is>
+      </c>
+      <c r="C2239" s="0" t="inlineStr">
+        <is>
+          <t>sarva mangal, mangalya</t>
+        </is>
+      </c>
+      <c r="F2239" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 2 — shared aim of upasanas; मांगल्य abstract cognate.</t>
+        </is>
+      </c>
+      <c r="I2239" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" s="0" t="inlineStr">
+        <is>
+          <t>न्यूनातिरेक</t>
+        </is>
+      </c>
+      <c r="B2240" s="0" t="inlineStr">
+        <is>
+          <t>deficiency-or-excess</t>
+        </is>
+      </c>
+      <c r="C2240" s="0" t="inlineStr">
+        <is>
+          <t>nyoonatirek</t>
+        </is>
+      </c>
+      <c r="F2240" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 2 — न्यून + अतिरेक; faulty (imposed) self-evaluation.</t>
+        </is>
+      </c>
+      <c r="I2240" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" s="0" t="inlineStr">
+        <is>
+          <t>साम्राज्य</t>
+        </is>
+      </c>
+      <c r="B2241" s="0" t="inlineStr">
+        <is>
+          <t>dominion</t>
+        </is>
+      </c>
+      <c r="C2241" s="0" t="inlineStr">
+        <is>
+          <t>samrajya</t>
+        </is>
+      </c>
+      <c r="F2241" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 2 — "dominion" (not "sovereignty") to keep distinct from प्रभुसत्ता.</t>
+        </is>
+      </c>
+      <c r="I2241" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" s="0" t="inlineStr">
+        <is>
+          <t>पाण्डित्य</t>
+        </is>
+      </c>
+      <c r="B2242" s="0" t="inlineStr">
+        <is>
+          <t>scholarliness</t>
+        </is>
+      </c>
+      <c r="C2242" s="0" t="inlineStr">
+        <is>
+          <t>panditya</t>
+        </is>
+      </c>
+      <c r="F2242" s="0" t="inlineStr">
+        <is>
+          <t>KD glossary addition (2026-07): KD 2 — first KD appearance at p.31 (निपुणता एवं कुशलता, पाण्डित्य).</t>
+        </is>
+      </c>
+      <c r="I2242" s="0" t="inlineStr">
+        <is>
+          <t>KD-Glossary-Additions.md; KD 2</t>
         </is>
       </c>
     </row>
@@ -61618,12 +62563,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>worthiness</t>
+          <t>receptivity / worthiness (contextual)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
+          <t>CONTEXTUAL RULE (2026-07-10): in the क्षमता/योग्यता/पात्रता triad, use **receptivity** (aligned with MD-Mapping/MVD: capacity, ability, receptivity). Reserve **worthiness** for KD 3.10's technical contrast among दया/कृपा/करूणा (compassion/grace/mercy), where substances are made available "in accordance with worthiness (*patrata*)"</t>
         </is>
       </c>
     </row>
@@ -62696,12 +63641,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>the triad of desires</t>
+          <t>the "desires-trio"</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>KD 2: paired with विषय-चतुष्टय, tied to adhidaivik (social/behavioural) values. Not in MD-Mapping; left transliterated per the classical Sanskrit ऐषणा-त्रय (putra/vitta/loka-eshana), judgment call</t>
+          <t>KD 2: paired with विषय-चतुष्टय, tied to adhidaivik (social/behavioural) values. X-त्रय = "X-trio" (not "triad of X"), matching MVD/SB and the 2026-07-09 body convention. MD-Mapping has motive-trio; KD keeps "desires" for classical ऐषणा. Left transliterated (*eshana-traya*)</t>
         </is>
       </c>
     </row>
@@ -62806,12 +63751,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>the "triad of *-tā*"</t>
+          <t>the "*-tā*-trio"</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>KD 2 p.44: "स्वयं का मूल्यांकन 'ता-त्रय' की सीमा में होता है" (self-evaluation occurs within the domain of the tā-traya). UNCERTAIN — not in MD-Mapping; the surrounding text repeatedly pairs क्षमता/योग्यता/पात्रता (capacity/competence/worthiness), which is the likeliest referent, but the source does not gloss the compound explicitly here. Left transliterated and flagged for human review rather than asserted</t>
+          <t>KD 2 p.44: "स्वयं का मूल्यांकन 'ता-त्रय' की सीमा में होता है" (self-evaluation occurs within the domain of the tā-traya). UNCERTAIN — not in MD-Mapping; the surrounding text repeatedly pairs क्षमता/योग्यता/पात्रता (capacity/ability/receptivity), which is the likeliest referent, but the source does not gloss the compound explicitly here. Left transliterated and flagged for human review rather than asserted</t>
         </is>
       </c>
     </row>
@@ -63222,7 +64167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="114" min="1" max="1"/>
@@ -63882,12 +64827,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>worthiness</t>
+          <t>receptivity / worthiness (contextual)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>KD 3.10: the basis on which दया/कृपा/करूणा (compassion/grace/mercy) are distinguished — not in MD-Mapping under this exact sense, judgment call</t>
+          <t>CONTEXTUAL RULE (2026-07-10): in the क्षमता/योग्यता/पात्रता triad, use **receptivity** (aligned with MD-Mapping/MVD: capacity, ability, receptivity). Reserve **worthiness** for KD 3.10's technical contrast among दया/कृपा/करूणा (compassion/grace/mercy), where substances are made available "in accordance with worthiness (*patrata*)"</t>
         </is>
       </c>
     </row>
@@ -64576,284 +65521,482 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>निवृत्ति</t>
+          <t>मति</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Disencumberance, Disinclination</t>
+          <t>mati, sumati, anumati (left transliterated)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>disencumberance</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
+          <t>KD 1: triad of "righteous-action-born intellect" (सुकर्म-जन्य-बुद्धि), not in MD-Mapping; left transliterated, glossed in-text</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>सुमति</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>cause</t>
+          <t>mati, sumati, anumati (left transliterated)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>gross, subtle, causal</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
+          <t>KD 1: triad of "righteous-action-born intellect" (सुकर्म-जन्य-बुद्धि), not in MD-Mapping; left transliterated, glossed in-text</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>उपासना</t>
+          <t>अनुमति</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>worship, upasana</t>
+          <t>mati, sumati, anumati (left transliterated)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Upasana (worship)</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
+          <t>KD 1: triad of "righteous-action-born intellect" (सुकर्म-जन्य-बुद्धि), not in MD-Mapping; left transliterated, glossed in-text</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>नश्वरत्व</t>
+          <t>अमति</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>mortality</t>
+          <t>amati, kumati, durmati (left transliterated)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>perishability</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
+          <t>KD 1: triad of "unrighteous-action-born tendency" (दुष्कर्म-जन्य-प्रवृत्ति), parallel to मति/सुमति/अनुमति; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>देवात्मा</t>
+          <t>कुमति</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>deific-self</t>
+          <t>amati, kumati, durmati (left transliterated)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>the deific soul, the elemental soul, the divine soul</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+          <t>KD 1: triad of "unrighteous-action-born tendency" (दुष्कर्म-जन्य-प्रवृत्ति), parallel to मति/सुमति/अनुमति; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>दिव्यात्मा</t>
+          <t>दुर्मति</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>divine-self</t>
+          <t>amati, kumati, durmati (left transliterated)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>the deific soul, the elemental soul, the divine soul</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+          <t>KD 1: triad of "unrighteous-action-born tendency" (दुष्कर्म-जन्य-प्रवृत्ति), parallel to मति/सुमति/अनुमति; not in MD-Mapping</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>विद्या</t>
+          <t>निवृत्ति</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>Disencumberance, Disinclination</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>learning, sub-learning, base learning</t>
+          <t>disencumberance</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
+          <t>Per MD-Mapping ("Disencumberance, Disinclination" — freedom from delusion, fear, bondage). KD 1: one link in a definitional chain (ascertainment → disencumberance → impetus/wisdom → ...)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>तदाकार</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>absolute-resonance</t>
+          <t>cause</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>taking-the-form-of</t>
+          <t>gross, subtle, causal</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
+          <t>KD 1: classical triad (not in MD-Mapping under this exact grouping) for the three levels at which direct-perception, inference, and testimony-activity, and independent/imitative/adherent tendency, all operate</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>वर्ग</t>
+          <t>रजोगुण</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>class</t>
+          <t>rajoguna, tamoguna, sattvaguna (left transliterated)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>creed, sect, class</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>KD 2 p.38: "मानव के स्वधर्म में ही मत, सम्प्रदाय, वर्ग तिरोहित हो जाते हैं" — not in MD-Mapping under this triad, compositional</t>
+          <t>KD 1: the classical three गुण (property-modes), mapped onto sam/visham/mediating (see सम-विषम-मध्यस्थ row above: sam=rajoguna, visham=tamoguna, mediating=sattvaguna); not in MD-Mapping, kept transliterated per standard practice for this well-known Sanskrit triad</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>अभ्युदय</t>
+          <t>तमोगुण</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>comprehensive resolution (Abhyudaya)</t>
+          <t>rajoguna, tamoguna, sattvaguna (left transliterated)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>comprehensive resolution</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
+          <t>KD 1: the classical three गुण (property-modes), mapped onto sam/visham/mediating (see सम-विषम-मध्यस्थ row above: sam=rajoguna, visham=tamoguna, mediating=sattvaguna); not in MD-Mapping, kept transliterated per standard practice for this well-known Sanskrit triad</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>प्रभुसत्ता</t>
+          <t>सत्वगुण</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Supreme order</t>
+          <t>rajoguna, tamoguna, sattvaguna (left transliterated)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>sovereignty</t>
+          <t>left transliterated</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
+          <t>KD 1: the classical three गुण (property-modes), mapped onto sam/visham/mediating (see सम-विषम-मध्यस्थ row above: sam=rajoguna, visham=tamoguna, mediating=sattvaguna); not in MD-Mapping, kept transliterated per standard practice for this well-known Sanskrit triad</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>वैराग्य</t>
+          <t>उपासना</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>detachment</t>
+          <t>worship, upasana</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>dispassion</t>
+          <t>Upasana (worship)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+          <t>KD 2 chapter title. Per MD-Mapping ("worship, upasana") and SB's own English rendering (SB p.23: "worship, archana, yoga, sadhana, and upasana" — SB itself leaves उपासना transliterated rather than translating it). Kept transliterated as "upasana" throughout, glossed "(worship)" on first use, per this project's practice for the book's central chapter-2 term</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>नश्वरत्व</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>mortality</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>perishability</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>KD 2 opening line, contrasted with अमरत्व (immortality) — "जीवन के अमरत्व, शरीर के नश्वरत्व" → "the immortality of jeevan, the perishability of the body"; not in MD-Mapping, compositional judgment call</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>देवात्मा</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>deific-self</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>the deific soul, the elemental soul, the divine soul</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>दिव्यात्मा</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>divine-self</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>the deific soul, the elemental soul, the divine soul</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>KD 2: the three states of soul, tied to absolute-oneness (*tadatmya*) with, respectively, adhidaivik facts, adhibhautik elements, and the Spirit (adhyatma) — parallels the established अधिदैवीवाद/अधिभौतिकवाद/अध्यात्मवाद triad (KD 3.17 glossary row). देवात्मा = "deific-self" per MD-Mapping, rendered "deific soul" here for parallelism with the other two (compositional; MD-Mapping does not carry भूतात्मा/दिव्यात्मा)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>विद्या</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>learning</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>learning, sub-learning, base learning</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>KD 2: the three qualities of upasana outcome, tied respectively to divine, deific, and elemental souls. विद्या = "learning" per MD-Mapping; उपविद्या and क्षुद्र विद्या are KD coinages not in MD-Mapping, compositional (उप- = sub-, क्षुद्र = base/petty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>तदाकार</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>absolute-resonance</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>taking-the-form-of</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>KD 2 p.40: recurring construction ("जल में तदाकार होने से..." = "by taking-the-form-of water...") applied to water, fire, air, light; compositional (तत् + आकार), not in MD-Mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>वर्ग</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>creed, sect, class</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>KD 2 p.38: "मानव के स्वधर्म में ही मत, सम्प्रदाय, वर्ग तिरोहित हो जाते हैं" — not in MD-Mapping under this triad, compositional</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>अभ्युदय</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>comprehensive resolution (Abhyudaya)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>comprehensive resolution</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Settled per Raghava (2026-07-08), aligned with MVD p.23 (supersedes "well-being" / "rise"); KD 2 p.35 and KD 3.12 p.116 in KD-Karm-Darshan-English.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>प्रभुसत्ता</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Supreme order</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>sovereignty</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>KD 2 p.41: प्रभु (lord/sovereign) + सत्ता; kept distinct from साम्राज्य (below) to avoid collision</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>वैराग्य</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>detachment</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>dispassion</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Both established as "dispassion," consistent with KD 1's अनासक्ति = "dispassion" (ch1 glossary note); KD 2 pp.48–49 uses विराग and its classical synonym वैराग्य side by side in a causal chain (विराग → आत्म-लक्ष्य; आत्म-प्रतिष्ठा → पर-वैराग्य)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
           <t>अवकाश</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>void</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>opportunity</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>Settled per Raghava (2026-07-09): **not** "leisure." KD 1 p.14 (PDF p.39) glosses अवकाश (सम्भावना) → "opportunity (possibility)"; body/mind/wealth as means is itself opportunity; paired with अवसर ("occasion") in "necessity, occasion, and opportunity." Distinct from MD-Mapping's आकाश, अवकाश = "void" (space sense). MVD renders अवकाश एवम् अवसर as "opportunity and scope"</t>
         </is>

</xml_diff>